<commit_message>
feat(schema): split dpv core into eigth semantic sub-schemas
</commit_message>
<xml_diff>
--- a/project/excel/dpv.xlsx
+++ b/project/excel/dpv.xlsx
@@ -7,978 +7,978 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AIGovernance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AILiteracy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AINotice" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AcademicResearch" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="AcademicScientificOrganisation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="AcceptContract" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="AcceptableRule" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="AcceptableUsePolicy" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Access" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="AccessControlMethod" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="AccountManagement" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Acquire" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ActiveRight" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="ActivelyInvolved" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="ActivityCompleted" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ActivityHalted" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ActivityMonitoring" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="ActivityNotCompleted" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="ActivityOngoing" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="ActivityPlanned" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="ActivityProposed" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="ActivityStatus" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Adapt" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Adult" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Advertising" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="AgeVerification" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Aggregate" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="AlgorithmicLogic" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Align" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Alter" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="AmbulanceProvider" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="Analyse" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="Anonymisation" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="Anonymise" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="AnonymisedData" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="Applicability" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="Applicant" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="ApprovalProcedure" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="Assess" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="Assessment" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="AssetManagementProcedures" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="AssistiveAutomation" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="AsylumSeeker" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="AsymmetricCryptography" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="AsymmetricEncryption" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="Audit" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="AuditApproved" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="AuditConditionallyApproved" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="AuditNotRequired" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="AuditRejected" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="AuditRequested" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="AuditRequired" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="AuditStatus" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="AuthenticationABC" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="AuthenticationPABC" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="AuthenticationProtocols" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="AuthorisationProcedure" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="AuthorisationProtocols" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="AuthorityInformed" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="AuthorityUninformed" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="AutomatedDecisionMaking" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="AutomatedScoringOfIndividuals" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="AutomationLevel" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="Autonomous" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="B2B2CContract" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="B2BContract" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="B2CContract" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="BackgroundChecks" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="BiometricAuthentication" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="C2BContract" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="C2CContract" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="CannotChallengeProcess" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="CannotChallengeProcessInput" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="CannotChallengeProcessOutput" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="CannotCorrectProcess" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="CannotCorrectProcessInput" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="CannotCorrectProcessOutput" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="CannotObjectToProcess" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="CannotOptInToProcess" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="CannotOptOutFromProcess" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet name="CannotReverseProcessEffects" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet name="CannotReverseProcessInput" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet name="CannotReverseProcessOutput" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet name="CannotWithdrawFromProcess" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet name="Certification" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet name="CertificationSeal" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet name="ChallengingProcess" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet name="ChallengingProcessInput" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet name="ChallengingProcessOutput" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet name="CharityOrganisation" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet name="Child" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet name="Citizen" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet name="City" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet name="Client" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet name="Clinic" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet name="CloudLocation" sheetId="96" state="visible" r:id="rId96"/>
-    <sheet name="CodeOfConduct" sheetId="97" state="visible" r:id="rId97"/>
-    <sheet name="Collect" sheetId="98" state="visible" r:id="rId98"/>
-    <sheet name="CollectedData" sheetId="99" state="visible" r:id="rId99"/>
-    <sheet name="CollectedPersonalData" sheetId="100" state="visible" r:id="rId100"/>
-    <sheet name="CombatClimateChange" sheetId="101" state="visible" r:id="rId101"/>
-    <sheet name="Combine" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet name="CommercialPurpose" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet name="CommercialResearch" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet name="CommerciallyConfidentialData" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet name="CommunicationForCustomerCare" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet name="CommunicationManagement" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet name="CompatibilityUnknown" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet name="ComplianceAssessment" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet name="ComplianceIndeterminate" sheetId="110" state="visible" r:id="rId110"/>
-    <sheet name="ComplianceMonitoring" sheetId="111" state="visible" r:id="rId111"/>
-    <sheet name="ComplianceStatus" sheetId="112" state="visible" r:id="rId112"/>
-    <sheet name="ComplianceUnknown" sheetId="113" state="visible" r:id="rId113"/>
-    <sheet name="ComplianceViolation" sheetId="114" state="visible" r:id="rId114"/>
-    <sheet name="Compliant" sheetId="115" state="visible" r:id="rId115"/>
-    <sheet name="ConditionalAutomation" sheetId="116" state="visible" r:id="rId116"/>
-    <sheet name="ConfidentialData" sheetId="117" state="visible" r:id="rId117"/>
-    <sheet name="ConfidentialityAgreement" sheetId="118" state="visible" r:id="rId118"/>
-    <sheet name="ConformanceAssessment" sheetId="119" state="visible" r:id="rId119"/>
-    <sheet name="ConformanceStatus" sheetId="120" state="visible" r:id="rId120"/>
-    <sheet name="Conformant" sheetId="121" state="visible" r:id="rId121"/>
-    <sheet name="Consent" sheetId="122" state="visible" r:id="rId122"/>
-    <sheet name="ConsentControl" sheetId="123" state="visible" r:id="rId123"/>
-    <sheet name="ConsentExpired" sheetId="124" state="visible" r:id="rId124"/>
-    <sheet name="ConsentGiven" sheetId="125" state="visible" r:id="rId125"/>
-    <sheet name="ConsentInvalidated" sheetId="126" state="visible" r:id="rId126"/>
-    <sheet name="ConsentManagement" sheetId="127" state="visible" r:id="rId127"/>
-    <sheet name="ConsentNotice" sheetId="128" state="visible" r:id="rId128"/>
-    <sheet name="ConsentReceipt" sheetId="129" state="visible" r:id="rId129"/>
-    <sheet name="ConsentRecord" sheetId="130" state="visible" r:id="rId130"/>
-    <sheet name="ConsentRefused" sheetId="131" state="visible" r:id="rId131"/>
-    <sheet name="ConsentRequestDeferred" sheetId="132" state="visible" r:id="rId132"/>
-    <sheet name="ConsentRequested" sheetId="133" state="visible" r:id="rId133"/>
-    <sheet name="ConsentRevoked" sheetId="134" state="visible" r:id="rId134"/>
-    <sheet name="ConsentStatus" sheetId="135" state="visible" r:id="rId135"/>
-    <sheet name="ConsentStatusInvalidForProcessing" sheetId="136" state="visible" r:id="rId136"/>
-    <sheet name="ConsentStatusValidForProcessing" sheetId="137" state="visible" r:id="rId137"/>
-    <sheet name="ConsentUnknown" sheetId="138" state="visible" r:id="rId138"/>
-    <sheet name="ConsentWithdrawn" sheetId="139" state="visible" r:id="rId139"/>
-    <sheet name="Consequence" sheetId="140" state="visible" r:id="rId140"/>
-    <sheet name="ConsequenceAsSideEffect" sheetId="141" state="visible" r:id="rId141"/>
-    <sheet name="ConsequenceOfFailure" sheetId="142" state="visible" r:id="rId142"/>
-    <sheet name="ConsequenceOfSuccess" sheetId="143" state="visible" r:id="rId143"/>
-    <sheet name="Consult" sheetId="144" state="visible" r:id="rId144"/>
-    <sheet name="Consultation" sheetId="145" state="visible" r:id="rId145"/>
-    <sheet name="ConsultationWithAuthority" sheetId="146" state="visible" r:id="rId146"/>
-    <sheet name="ConsultationWithDPO" sheetId="147" state="visible" r:id="rId147"/>
-    <sheet name="ConsultationWithDataSubject" sheetId="148" state="visible" r:id="rId148"/>
-    <sheet name="ConsultationWithDataSubjectRepresentative" sheetId="149" state="visible" r:id="rId149"/>
-    <sheet name="ConsumerStandardFormContract" sheetId="150" state="visible" r:id="rId150"/>
-    <sheet name="Context" sheetId="151" state="visible" r:id="rId151"/>
-    <sheet name="ContextuallyAnonymisedData" sheetId="152" state="visible" r:id="rId152"/>
-    <sheet name="ContinuousFrequency" sheetId="153" state="visible" r:id="rId153"/>
-    <sheet name="Contract" sheetId="154" state="visible" r:id="rId154"/>
-    <sheet name="ContractActivationStatus" sheetId="155" state="visible" r:id="rId155"/>
-    <sheet name="ContractActive" sheetId="156" state="visible" r:id="rId156"/>
-    <sheet name="ContractAmended" sheetId="157" state="visible" r:id="rId157"/>
-    <sheet name="ContractAmendmentClause" sheetId="158" state="visible" r:id="rId158"/>
-    <sheet name="ContractApproved" sheetId="159" state="visible" r:id="rId159"/>
-    <sheet name="ContractBeingPerformed" sheetId="160" state="visible" r:id="rId160"/>
-    <sheet name="ContractBreached" sheetId="161" state="visible" r:id="rId161"/>
-    <sheet name="ContractByDomain" sheetId="162" state="visible" r:id="rId162"/>
-    <sheet name="ContractByEntityType" sheetId="163" state="visible" r:id="rId163"/>
-    <sheet name="ContractByNegotiationType" sheetId="164" state="visible" r:id="rId164"/>
-    <sheet name="ContractConfidentialityClause" sheetId="165" state="visible" r:id="rId165"/>
-    <sheet name="ContractControl" sheetId="166" state="visible" r:id="rId166"/>
-    <sheet name="ContractDefinitions" sheetId="167" state="visible" r:id="rId167"/>
-    <sheet name="ContractDisputeResolutionClause" sheetId="168" state="visible" r:id="rId168"/>
-    <sheet name="ContractDisputed" sheetId="169" state="visible" r:id="rId169"/>
-    <sheet name="ContractDrafted" sheetId="170" state="visible" r:id="rId170"/>
-    <sheet name="ContractExecutionStatus" sheetId="171" state="visible" r:id="rId171"/>
-    <sheet name="ContractExpired" sheetId="172" state="visible" r:id="rId172"/>
-    <sheet name="ContractExtended" sheetId="173" state="visible" r:id="rId173"/>
-    <sheet name="ContractFulfilled" sheetId="174" state="visible" r:id="rId174"/>
-    <sheet name="ContractFulfilmentStatus" sheetId="175" state="visible" r:id="rId175"/>
-    <sheet name="ContractFullyExecuted" sheetId="176" state="visible" r:id="rId176"/>
-    <sheet name="ContractFullySigned" sheetId="177" state="visible" r:id="rId177"/>
-    <sheet name="ContractInactive" sheetId="178" state="visible" r:id="rId178"/>
-    <sheet name="ContractJurisdictionClause" sheetId="179" state="visible" r:id="rId179"/>
-    <sheet name="ContractNegotiated" sheetId="180" state="visible" r:id="rId180"/>
-    <sheet name="ContractNotFulfilled" sheetId="181" state="visible" r:id="rId181"/>
-    <sheet name="ContractOffered" sheetId="182" state="visible" r:id="rId182"/>
-    <sheet name="ContractPartiallyFulfilled" sheetId="183" state="visible" r:id="rId183"/>
-    <sheet name="ContractPartiallySigned" sheetId="184" state="visible" r:id="rId184"/>
-    <sheet name="ContractPerformance" sheetId="185" state="visible" r:id="rId185"/>
-    <sheet name="ContractPerformanceStatus" sheetId="186" state="visible" r:id="rId186"/>
-    <sheet name="ContractPreamble" sheetId="187" state="visible" r:id="rId187"/>
-    <sheet name="ContractPreparationStatus" sheetId="188" state="visible" r:id="rId188"/>
-    <sheet name="ContractRejected" sheetId="189" state="visible" r:id="rId189"/>
-    <sheet name="ContractRenewed" sheetId="190" state="visible" r:id="rId190"/>
-    <sheet name="ContractSignedByParty" sheetId="191" state="visible" r:id="rId191"/>
-    <sheet name="ContractStatus" sheetId="192" state="visible" r:id="rId192"/>
-    <sheet name="ContractTemporarilySuspended" sheetId="193" state="visible" r:id="rId193"/>
-    <sheet name="ContractTerminated" sheetId="194" state="visible" r:id="rId194"/>
-    <sheet name="ContractTerminationClause" sheetId="195" state="visible" r:id="rId195"/>
-    <sheet name="ContractTerminationStatus" sheetId="196" state="visible" r:id="rId196"/>
-    <sheet name="ContractUnderNegotiation" sheetId="197" state="visible" r:id="rId197"/>
-    <sheet name="ContractUnderReview" sheetId="198" state="visible" r:id="rId198"/>
-    <sheet name="ContractViolated" sheetId="199" state="visible" r:id="rId199"/>
-    <sheet name="ContractualClause" sheetId="200" state="visible" r:id="rId200"/>
-    <sheet name="ContractualClauseFulfilled" sheetId="201" state="visible" r:id="rId201"/>
-    <sheet name="ContractualClauseFulfilmentStatus" sheetId="202" state="visible" r:id="rId202"/>
-    <sheet name="ContractualClauseNotFulfilled" sheetId="203" state="visible" r:id="rId203"/>
-    <sheet name="ContractualClausePartiallyFulfilled" sheetId="204" state="visible" r:id="rId204"/>
-    <sheet name="ContractualClauseViolated" sheetId="205" state="visible" r:id="rId205"/>
-    <sheet name="ContractualTerms" sheetId="206" state="visible" r:id="rId206"/>
-    <sheet name="ControllerDataSubjectAgreement" sheetId="207" state="visible" r:id="rId207"/>
-    <sheet name="ControllerInformed" sheetId="208" state="visible" r:id="rId208"/>
-    <sheet name="ControllerProcessorAgreement" sheetId="209" state="visible" r:id="rId209"/>
-    <sheet name="ControllerUninformed" sheetId="210" state="visible" r:id="rId210"/>
-    <sheet name="Copy" sheetId="211" state="visible" r:id="rId211"/>
-    <sheet name="CorrectingProcess" sheetId="212" state="visible" r:id="rId212"/>
-    <sheet name="CorrectingProcessInput" sheetId="213" state="visible" r:id="rId213"/>
-    <sheet name="CorrectingProcessOutput" sheetId="214" state="visible" r:id="rId214"/>
-    <sheet name="CounterMoneyLaundering" sheetId="215" state="visible" r:id="rId215"/>
-    <sheet name="Counterterrorism" sheetId="216" state="visible" r:id="rId216"/>
-    <sheet name="CredentialManagement" sheetId="217" state="visible" r:id="rId217"/>
-    <sheet name="CrossBorderTransfer" sheetId="218" state="visible" r:id="rId218"/>
-    <sheet name="CryptographicAuthentication" sheetId="219" state="visible" r:id="rId219"/>
-    <sheet name="CryptographicKeyManagement" sheetId="220" state="visible" r:id="rId220"/>
-    <sheet name="CryptographicMethods" sheetId="221" state="visible" r:id="rId221"/>
-    <sheet name="CustomerCare" sheetId="222" state="visible" r:id="rId222"/>
-    <sheet name="CustomerClaimsManagement" sheetId="223" state="visible" r:id="rId223"/>
-    <sheet name="CustomerManagement" sheetId="224" state="visible" r:id="rId224"/>
-    <sheet name="CustomerOrderManagement" sheetId="225" state="visible" r:id="rId225"/>
-    <sheet name="CustomerRelationshipManagement" sheetId="226" state="visible" r:id="rId226"/>
-    <sheet name="CustomerSolvencyMonitoring" sheetId="227" state="visible" r:id="rId227"/>
-    <sheet name="CybersecurityAssessment" sheetId="228" state="visible" r:id="rId228"/>
-    <sheet name="CybersecurityTraining" sheetId="229" state="visible" r:id="rId229"/>
-    <sheet name="DPIA" sheetId="230" state="visible" r:id="rId230"/>
-    <sheet name="DashboardNotice" sheetId="231" state="visible" r:id="rId231"/>
-    <sheet name="DataAltruism" sheetId="232" state="visible" r:id="rId232"/>
-    <sheet name="DataAvailabilityAssessment" sheetId="233" state="visible" r:id="rId233"/>
-    <sheet name="DataBackupProtocols" sheetId="234" state="visible" r:id="rId234"/>
-    <sheet name="DataBreachImpactAssessment" sheetId="235" state="visible" r:id="rId235"/>
-    <sheet name="DataBreachNotice" sheetId="236" state="visible" r:id="rId236"/>
-    <sheet name="DataBreachNotification" sheetId="237" state="visible" r:id="rId237"/>
-    <sheet name="DataBreachRecord" sheetId="238" state="visible" r:id="rId238"/>
-    <sheet name="DataController" sheetId="239" state="visible" r:id="rId239"/>
-    <sheet name="DataControllerContract" sheetId="240" state="visible" r:id="rId240"/>
-    <sheet name="DataControllerDataSource" sheetId="241" state="visible" r:id="rId241"/>
-    <sheet name="DataDeletionPolicy" sheetId="242" state="visible" r:id="rId242"/>
-    <sheet name="DataErasurePolicy" sheetId="243" state="visible" r:id="rId243"/>
-    <sheet name="DataExporter" sheetId="244" state="visible" r:id="rId244"/>
-    <sheet name="DataGovernance" sheetId="245" state="visible" r:id="rId245"/>
-    <sheet name="DataHandlingClause" sheetId="246" state="visible" r:id="rId246"/>
-    <sheet name="DataImporter" sheetId="247" state="visible" r:id="rId247"/>
-    <sheet name="DataInteroperabilityAssessment" sheetId="248" state="visible" r:id="rId248"/>
-    <sheet name="DataInteroperabilityImprovement" sheetId="249" state="visible" r:id="rId249"/>
-    <sheet name="DataInteroperabilityManagement" sheetId="250" state="visible" r:id="rId250"/>
-    <sheet name="DataInventoryManagement" sheetId="251" state="visible" r:id="rId251"/>
-    <sheet name="DataJurisdictionPolicy" sheetId="252" state="visible" r:id="rId252"/>
-    <sheet name="DataLiteracy" sheetId="253" state="visible" r:id="rId253"/>
-    <sheet name="DataProcessingAgreement" sheetId="254" state="visible" r:id="rId254"/>
-    <sheet name="DataProcessingPolicy" sheetId="255" state="visible" r:id="rId255"/>
-    <sheet name="DataProcessingRecord" sheetId="256" state="visible" r:id="rId256"/>
-    <sheet name="DataProcessor" sheetId="257" state="visible" r:id="rId257"/>
-    <sheet name="DataProcessorContract" sheetId="258" state="visible" r:id="rId258"/>
-    <sheet name="DataProtectionAuthority" sheetId="259" state="visible" r:id="rId259"/>
-    <sheet name="DataProtectionOfficer" sheetId="260" state="visible" r:id="rId260"/>
-    <sheet name="DataProtectionTraining" sheetId="261" state="visible" r:id="rId261"/>
-    <sheet name="DataPublishedByDataSubject" sheetId="262" state="visible" r:id="rId262"/>
-    <sheet name="DataQualityAssessment" sheetId="263" state="visible" r:id="rId263"/>
-    <sheet name="DataQualityImprovement" sheetId="264" state="visible" r:id="rId264"/>
-    <sheet name="DataQualityManagement" sheetId="265" state="visible" r:id="rId265"/>
-    <sheet name="DataRedaction" sheetId="266" state="visible" r:id="rId266"/>
-    <sheet name="DataRestorationPolicy" sheetId="267" state="visible" r:id="rId267"/>
-    <sheet name="DataReusePolicy" sheetId="268" state="visible" r:id="rId268"/>
-    <sheet name="DataSanitisationTechnique" sheetId="269" state="visible" r:id="rId269"/>
-    <sheet name="DataSecurityManagement" sheetId="270" state="visible" r:id="rId270"/>
-    <sheet name="DataSource" sheetId="271" state="visible" r:id="rId271"/>
-    <sheet name="DataStoragePolicy" sheetId="272" state="visible" r:id="rId272"/>
-    <sheet name="DataSubProcessor" sheetId="273" state="visible" r:id="rId273"/>
-    <sheet name="DataSubject" sheetId="274" state="visible" r:id="rId274"/>
-    <sheet name="DataSubjectContract" sheetId="275" state="visible" r:id="rId275"/>
-    <sheet name="DataSubjectDataSource" sheetId="276" state="visible" r:id="rId276"/>
-    <sheet name="DataSubjectInformed" sheetId="277" state="visible" r:id="rId277"/>
-    <sheet name="DataSubjectRight" sheetId="278" state="visible" r:id="rId278"/>
-    <sheet name="DataSubjectRightsManagement" sheetId="279" state="visible" r:id="rId279"/>
-    <sheet name="DataSubjectScale" sheetId="280" state="visible" r:id="rId280"/>
-    <sheet name="DataSubjectUninformed" sheetId="281" state="visible" r:id="rId281"/>
-    <sheet name="DataSuitabilityAssessment" sheetId="282" state="visible" r:id="rId282"/>
-    <sheet name="DataTransferImpactAssessment" sheetId="283" state="visible" r:id="rId283"/>
-    <sheet name="DataTransferLegalBasis" sheetId="284" state="visible" r:id="rId284"/>
-    <sheet name="DataTransferNotice" sheetId="285" state="visible" r:id="rId285"/>
-    <sheet name="DataTransferRecord" sheetId="286" state="visible" r:id="rId286"/>
-    <sheet name="DataVolume" sheetId="287" state="visible" r:id="rId287"/>
-    <sheet name="DecentralisedLocations" sheetId="288" state="visible" r:id="rId288"/>
-    <sheet name="DecisionMaking" sheetId="289" state="visible" r:id="rId289"/>
-    <sheet name="Deidentification" sheetId="290" state="visible" r:id="rId290"/>
-    <sheet name="Delete" sheetId="291" state="visible" r:id="rId291"/>
-    <sheet name="DeliveryOfGoods" sheetId="292" state="visible" r:id="rId292"/>
-    <sheet name="Derive" sheetId="293" state="visible" r:id="rId293"/>
-    <sheet name="DerivedData" sheetId="294" state="visible" r:id="rId294"/>
-    <sheet name="DerivedPersonalData" sheetId="295" state="visible" r:id="rId295"/>
-    <sheet name="DesignStandard" sheetId="296" state="visible" r:id="rId296"/>
-    <sheet name="Destruct" sheetId="297" state="visible" r:id="rId297"/>
-    <sheet name="DeterministicPseudonymisation" sheetId="298" state="visible" r:id="rId298"/>
-    <sheet name="Deterrence" sheetId="299" state="visible" r:id="rId299"/>
-    <sheet name="DeterrenceFollowed" sheetId="300" state="visible" r:id="rId300"/>
-    <sheet name="DeterrenceNotFollowed" sheetId="301" state="visible" r:id="rId301"/>
-    <sheet name="DeviceNotice" sheetId="302" state="visible" r:id="rId302"/>
-    <sheet name="DifferentialPrivacy" sheetId="303" state="visible" r:id="rId303"/>
-    <sheet name="DigitalLiteracy" sheetId="304" state="visible" r:id="rId304"/>
-    <sheet name="DigitalRightsManagement" sheetId="305" state="visible" r:id="rId305"/>
-    <sheet name="DigitalSignatures" sheetId="306" state="visible" r:id="rId306"/>
-    <sheet name="DirectMarketing" sheetId="307" state="visible" r:id="rId307"/>
-    <sheet name="DisasterRecoveryProcedures" sheetId="308" state="visible" r:id="rId308"/>
-    <sheet name="Disclose" sheetId="309" state="visible" r:id="rId309"/>
-    <sheet name="DiscloseByTransmission" sheetId="310" state="visible" r:id="rId310"/>
-    <sheet name="Display" sheetId="311" state="visible" r:id="rId311"/>
-    <sheet name="DisputeManagement" sheetId="312" state="visible" r:id="rId312"/>
-    <sheet name="Disseminate" sheetId="313" state="visible" r:id="rId313"/>
-    <sheet name="DistributedSystemSecurity" sheetId="314" state="visible" r:id="rId314"/>
-    <sheet name="DistributionAgreement" sheetId="315" state="visible" r:id="rId315"/>
-    <sheet name="DocumentRandomisedPseudonymisation" sheetId="316" state="visible" r:id="rId316"/>
-    <sheet name="DocumentSecurity" sheetId="317" state="visible" r:id="rId317"/>
-    <sheet name="Download" sheetId="318" state="visible" r:id="rId318"/>
-    <sheet name="DpvAgent" sheetId="319" state="visible" r:id="rId319"/>
-    <sheet name="DpvAuthority" sheetId="320" state="visible" r:id="rId320"/>
-    <sheet name="DpvConsumer" sheetId="321" state="visible" r:id="rId321"/>
-    <sheet name="DpvCountry" sheetId="322" state="visible" r:id="rId322"/>
-    <sheet name="DpvCustomer" sheetId="323" state="visible" r:id="rId323"/>
-    <sheet name="DpvData" sheetId="324" state="visible" r:id="rId324"/>
-    <sheet name="DpvDuration" sheetId="325" state="visible" r:id="rId325"/>
-    <sheet name="DpvEntity" sheetId="326" state="visible" r:id="rId326"/>
-    <sheet name="DpvJurisdiction" sheetId="327" state="visible" r:id="rId327"/>
-    <sheet name="DpvLocation" sheetId="328" state="visible" r:id="rId328"/>
-    <sheet name="DpvOptional" sheetId="329" state="visible" r:id="rId329"/>
-    <sheet name="DpvOrganisation" sheetId="330" state="visible" r:id="rId330"/>
-    <sheet name="DpvProcess" sheetId="331" state="visible" r:id="rId331"/>
-    <sheet name="DpvRecipient" sheetId="332" state="visible" r:id="rId332"/>
-    <sheet name="DpvRecord" sheetId="333" state="visible" r:id="rId333"/>
-    <sheet name="DpvRegion" sheetId="334" state="visible" r:id="rId334"/>
-    <sheet name="DpvService" sheetId="335" state="visible" r:id="rId335"/>
-    <sheet name="DpvUser" sheetId="336" state="visible" r:id="rId336"/>
-    <sheet name="EULA" sheetId="337" state="visible" r:id="rId337"/>
-    <sheet name="EconomicUnion" sheetId="338" state="visible" r:id="rId338"/>
-    <sheet name="EducationalOrganisation" sheetId="339" state="visible" r:id="rId339"/>
-    <sheet name="EducationalTraining" sheetId="340" state="visible" r:id="rId340"/>
-    <sheet name="EffectivenessDeterminationProcedures" sheetId="341" state="visible" r:id="rId341"/>
-    <sheet name="ElderlyDataSubject" sheetId="342" state="visible" r:id="rId342"/>
-    <sheet name="ElderlyHuman" sheetId="343" state="visible" r:id="rId343"/>
-    <sheet name="EmergencyHealthcareProvider" sheetId="344" state="visible" r:id="rId344"/>
-    <sheet name="EmergencyServiceProvider" sheetId="345" state="visible" r:id="rId345"/>
-    <sheet name="Employee" sheetId="346" state="visible" r:id="rId346"/>
-    <sheet name="EmploymentContract" sheetId="347" state="visible" r:id="rId347"/>
-    <sheet name="Encryption" sheetId="348" state="visible" r:id="rId348"/>
-    <sheet name="EncryptionAtRest" sheetId="349" state="visible" r:id="rId349"/>
-    <sheet name="EncryptionInTransfer" sheetId="350" state="visible" r:id="rId350"/>
-    <sheet name="EncryptionInUse" sheetId="351" state="visible" r:id="rId351"/>
-    <sheet name="EndToEndEncryption" sheetId="352" state="visible" r:id="rId352"/>
-    <sheet name="EndlessDuration" sheetId="353" state="visible" r:id="rId353"/>
-    <sheet name="EnforceAccessControl" sheetId="354" state="visible" r:id="rId354"/>
-    <sheet name="EnforceSecurity" sheetId="355" state="visible" r:id="rId355"/>
-    <sheet name="EnterIntoContract" sheetId="356" state="visible" r:id="rId356"/>
-    <sheet name="EntityActiveInvolvement" sheetId="357" state="visible" r:id="rId357"/>
-    <sheet name="EntityInformed" sheetId="358" state="visible" r:id="rId358"/>
-    <sheet name="EntityInformedStatus" sheetId="359" state="visible" r:id="rId359"/>
-    <sheet name="EntityIntendedInvolvement" sheetId="360" state="visible" r:id="rId360"/>
-    <sheet name="EntityInvolved" sheetId="361" state="visible" r:id="rId361"/>
-    <sheet name="EntityInvolvement" sheetId="362" state="visible" r:id="rId362"/>
-    <sheet name="EntityInvolvementStatus" sheetId="363" state="visible" r:id="rId363"/>
-    <sheet name="EntityNonInvolvement" sheetId="364" state="visible" r:id="rId364"/>
-    <sheet name="EntityNonPermissiveInvolvement" sheetId="365" state="visible" r:id="rId365"/>
-    <sheet name="EntityNotInvolved" sheetId="366" state="visible" r:id="rId366"/>
-    <sheet name="EntityPassiveInvolvement" sheetId="367" state="visible" r:id="rId367"/>
-    <sheet name="EntityPermissiveInvolvement" sheetId="368" state="visible" r:id="rId368"/>
-    <sheet name="EntityUninformed" sheetId="369" state="visible" r:id="rId369"/>
-    <sheet name="EntityUnintendedInvolvement" sheetId="370" state="visible" r:id="rId370"/>
-    <sheet name="EnvironmentalProtection" sheetId="371" state="visible" r:id="rId371"/>
-    <sheet name="Erase" sheetId="372" state="visible" r:id="rId372"/>
-    <sheet name="EstablishContractualAgreement" sheetId="373" state="visible" r:id="rId373"/>
-    <sheet name="EvaluationOfIndividuals" sheetId="374" state="visible" r:id="rId374"/>
-    <sheet name="EvaluationScoring" sheetId="375" state="visible" r:id="rId375"/>
-    <sheet name="ExpectationStatus" sheetId="376" state="visible" r:id="rId376"/>
-    <sheet name="Expected" sheetId="377" state="visible" r:id="rId377"/>
-    <sheet name="ExplicitlyExpressedConsent" sheetId="378" state="visible" r:id="rId378"/>
-    <sheet name="Export" sheetId="379" state="visible" r:id="rId379"/>
-    <sheet name="ExpressedConsent" sheetId="380" state="visible" r:id="rId380"/>
-    <sheet name="FRIA" sheetId="381" state="visible" r:id="rId381"/>
-    <sheet name="FailSafeProtocols" sheetId="382" state="visible" r:id="rId382"/>
-    <sheet name="FederatedLocations" sheetId="383" state="visible" r:id="rId383"/>
-    <sheet name="FeeNotRequired" sheetId="384" state="visible" r:id="rId384"/>
-    <sheet name="FeeRequired" sheetId="385" state="visible" r:id="rId385"/>
-    <sheet name="FeeRequirement" sheetId="386" state="visible" r:id="rId386"/>
-    <sheet name="FileSystemSecurity" sheetId="387" state="visible" r:id="rId387"/>
-    <sheet name="Filter" sheetId="388" state="visible" r:id="rId388"/>
-    <sheet name="FireDepartment" sheetId="389" state="visible" r:id="rId389"/>
-    <sheet name="FixedLocation" sheetId="390" state="visible" r:id="rId390"/>
-    <sheet name="FixedMultipleLocations" sheetId="391" state="visible" r:id="rId391"/>
-    <sheet name="FixedOccurrencesDuration" sheetId="392" state="visible" r:id="rId392"/>
-    <sheet name="FixedSingularLocation" sheetId="393" state="visible" r:id="rId393"/>
-    <sheet name="ForProfitOrganisation" sheetId="394" state="visible" r:id="rId394"/>
-    <sheet name="Format" sheetId="395" state="visible" r:id="rId395"/>
-    <sheet name="FraudPreventionAndDetection" sheetId="396" state="visible" r:id="rId396"/>
-    <sheet name="Frequency" sheetId="397" state="visible" r:id="rId397"/>
-    <sheet name="FulfilmentOfContractualObligation" sheetId="398" state="visible" r:id="rId398"/>
-    <sheet name="FulfilmentOfObligation" sheetId="399" state="visible" r:id="rId399"/>
-    <sheet name="FullAutomation" sheetId="400" state="visible" r:id="rId400"/>
-    <sheet name="FullyRandomisedPseudonymisation" sheetId="401" state="visible" r:id="rId401"/>
-    <sheet name="G2BContract" sheetId="402" state="visible" r:id="rId402"/>
-    <sheet name="G2CContract" sheetId="403" state="visible" r:id="rId403"/>
-    <sheet name="G2GContract" sheetId="404" state="visible" r:id="rId404"/>
-    <sheet name="Generate" sheetId="405" state="visible" r:id="rId405"/>
-    <sheet name="GeneratedData" sheetId="406" state="visible" r:id="rId406"/>
-    <sheet name="GeneratedPersonalData" sheetId="407" state="visible" r:id="rId407"/>
-    <sheet name="GeographicCoverage" sheetId="408" state="visible" r:id="rId408"/>
-    <sheet name="GlobalScale" sheetId="409" state="visible" r:id="rId409"/>
-    <sheet name="GovernanceProcedures" sheetId="410" state="visible" r:id="rId410"/>
-    <sheet name="GovernmentalOrganisation" sheetId="411" state="visible" r:id="rId411"/>
-    <sheet name="GraphicalNotice" sheetId="412" state="visible" r:id="rId412"/>
-    <sheet name="GuardianOfDataSubject" sheetId="413" state="visible" r:id="rId413"/>
-    <sheet name="GuardianOfHuman" sheetId="414" state="visible" r:id="rId414"/>
-    <sheet name="Guideline" sheetId="415" state="visible" r:id="rId415"/>
-    <sheet name="GuidelinesPrinciple" sheetId="416" state="visible" r:id="rId416"/>
-    <sheet name="HardwareSecurityProtocols" sheetId="417" state="visible" r:id="rId417"/>
-    <sheet name="HashFunctions" sheetId="418" state="visible" r:id="rId418"/>
-    <sheet name="HashMessageAuthenticationCode" sheetId="419" state="visible" r:id="rId419"/>
-    <sheet name="HealthcareOrganisation" sheetId="420" state="visible" r:id="rId420"/>
-    <sheet name="HighAutomation" sheetId="421" state="visible" r:id="rId421"/>
-    <sheet name="HomomorphicEncryption" sheetId="422" state="visible" r:id="rId422"/>
-    <sheet name="Hospital" sheetId="423" state="visible" r:id="rId423"/>
-    <sheet name="HugeDataVolume" sheetId="424" state="visible" r:id="rId424"/>
-    <sheet name="HugeScaleOfDataSubjects" sheetId="425" state="visible" r:id="rId425"/>
-    <sheet name="HumanInvolved" sheetId="426" state="visible" r:id="rId426"/>
-    <sheet name="HumanInvolvement" sheetId="427" state="visible" r:id="rId427"/>
-    <sheet name="HumanInvolvementForControl" sheetId="428" state="visible" r:id="rId428"/>
-    <sheet name="HumanInvolvementForDecision" sheetId="429" state="visible" r:id="rId429"/>
-    <sheet name="HumanInvolvementForInput" sheetId="430" state="visible" r:id="rId430"/>
-    <sheet name="HumanInvolvementForIntervention" sheetId="431" state="visible" r:id="rId431"/>
-    <sheet name="HumanInvolvementForOversight" sheetId="432" state="visible" r:id="rId432"/>
-    <sheet name="HumanInvolvementForVerification" sheetId="433" state="visible" r:id="rId433"/>
-    <sheet name="HumanNotInvolved" sheetId="434" state="visible" r:id="rId434"/>
-    <sheet name="HumanOversight" sheetId="435" state="visible" r:id="rId435"/>
-    <sheet name="HumanResourceManagement" sheetId="436" state="visible" r:id="rId436"/>
-    <sheet name="HumanSubject" sheetId="437" state="visible" r:id="rId437"/>
-    <sheet name="HybridPublicPrivateSpace" sheetId="438" state="visible" r:id="rId438"/>
-    <sheet name="IPRManagement" sheetId="439" state="visible" r:id="rId439"/>
-    <sheet name="IdentifyingPersonalData" sheetId="440" state="visible" r:id="rId440"/>
-    <sheet name="IdentityAuthentication" sheetId="441" state="visible" r:id="rId441"/>
-    <sheet name="IdentityManagementMethod" sheetId="442" state="visible" r:id="rId442"/>
-    <sheet name="IdentityVerification" sheetId="443" state="visible" r:id="rId443"/>
-    <sheet name="Immigrant" sheetId="444" state="visible" r:id="rId444"/>
-    <sheet name="Impact" sheetId="445" state="visible" r:id="rId445"/>
-    <sheet name="ImpactAssessment" sheetId="446" state="visible" r:id="rId446"/>
-    <sheet name="ImpliedConsent" sheetId="447" state="visible" r:id="rId447"/>
-    <sheet name="Importance" sheetId="448" state="visible" r:id="rId448"/>
-    <sheet name="ImproveExistingProductsAndServices" sheetId="449" state="visible" r:id="rId449"/>
-    <sheet name="ImproveHealthcare" sheetId="450" state="visible" r:id="rId450"/>
-    <sheet name="ImproveInternalCRMProcesses" sheetId="451" state="visible" r:id="rId451"/>
-    <sheet name="ImprovePublicServices" sheetId="452" state="visible" r:id="rId452"/>
-    <sheet name="ImproveTransportMobility" sheetId="453" state="visible" r:id="rId453"/>
-    <sheet name="IncidentManagementProcedures" sheetId="454" state="visible" r:id="rId454"/>
-    <sheet name="IncidentReportingCommunication" sheetId="455" state="visible" r:id="rId455"/>
-    <sheet name="IncorrectData" sheetId="456" state="visible" r:id="rId456"/>
-    <sheet name="IncreaseServiceRobustness" sheetId="457" state="visible" r:id="rId457"/>
-    <sheet name="IndeterminateDuration" sheetId="458" state="visible" r:id="rId458"/>
-    <sheet name="IndustryConsortium" sheetId="459" state="visible" r:id="rId459"/>
-    <sheet name="Infer" sheetId="460" state="visible" r:id="rId460"/>
-    <sheet name="InferredData" sheetId="461" state="visible" r:id="rId461"/>
-    <sheet name="InferredPersonalData" sheetId="462" state="visible" r:id="rId462"/>
-    <sheet name="InformationAudit" sheetId="463" state="visible" r:id="rId463"/>
-    <sheet name="InformationFlowControl" sheetId="464" state="visible" r:id="rId464"/>
-    <sheet name="InformationSecurityPolicy" sheetId="465" state="visible" r:id="rId465"/>
-    <sheet name="InformedConsent" sheetId="466" state="visible" r:id="rId466"/>
-    <sheet name="InnovativeUseOfExistingTechnology" sheetId="467" state="visible" r:id="rId467"/>
-    <sheet name="InnovativeUseOfNewTechnologies" sheetId="468" state="visible" r:id="rId468"/>
-    <sheet name="InnovativeUseOfTechnology" sheetId="469" state="visible" r:id="rId469"/>
-    <sheet name="IntellectualPropertyData" sheetId="470" state="visible" r:id="rId470"/>
-    <sheet name="Intended" sheetId="471" state="visible" r:id="rId471"/>
-    <sheet name="IntentionStatus" sheetId="472" state="visible" r:id="rId472"/>
-    <sheet name="InternalResourceOptimisation" sheetId="473" state="visible" r:id="rId473"/>
-    <sheet name="InternationalOrganisation" sheetId="474" state="visible" r:id="rId474"/>
-    <sheet name="IntrusionDetectionSystem" sheetId="475" state="visible" r:id="rId475"/>
-    <sheet name="InverseJurisdiction" sheetId="476" state="visible" r:id="rId476"/>
-    <sheet name="InvolvementStatus" sheetId="477" state="visible" r:id="rId477"/>
-    <sheet name="JITNotice" sheetId="478" state="visible" r:id="rId478"/>
-    <sheet name="JobApplicant" sheetId="479" state="visible" r:id="rId479"/>
-    <sheet name="JointDataControllers" sheetId="480" state="visible" r:id="rId480"/>
-    <sheet name="JointDataControllersAgreement" sheetId="481" state="visible" r:id="rId481"/>
-    <sheet name="JudicialOrganisation" sheetId="482" state="visible" r:id="rId482"/>
-    <sheet name="Justification" sheetId="483" state="visible" r:id="rId483"/>
-    <sheet name="LargeDataVolume" sheetId="484" state="visible" r:id="rId484"/>
-    <sheet name="LargeScaleOfDataSubjects" sheetId="485" state="visible" r:id="rId485"/>
-    <sheet name="LargeScaleProcessing" sheetId="486" state="visible" r:id="rId486"/>
-    <sheet name="Law" sheetId="487" state="visible" r:id="rId487"/>
-    <sheet name="LawEnforcementOrganisation" sheetId="488" state="visible" r:id="rId488"/>
-    <sheet name="Lawful" sheetId="489" state="visible" r:id="rId489"/>
-    <sheet name="Lawfulness" sheetId="490" state="visible" r:id="rId490"/>
-    <sheet name="LawfulnessUnknown" sheetId="491" state="visible" r:id="rId491"/>
-    <sheet name="LayeredNotice" sheetId="492" state="visible" r:id="rId492"/>
-    <sheet name="LegalAgent" sheetId="493" state="visible" r:id="rId493"/>
-    <sheet name="LegalAgreement" sheetId="494" state="visible" r:id="rId494"/>
-    <sheet name="LegalBasis" sheetId="495" state="visible" r:id="rId495"/>
-    <sheet name="LegalCompliance" sheetId="496" state="visible" r:id="rId496"/>
-    <sheet name="LegalComplianceAssessment" sheetId="497" state="visible" r:id="rId497"/>
-    <sheet name="LegalComplianceAudit" sheetId="498" state="visible" r:id="rId498"/>
-    <sheet name="LegalEntity" sheetId="499" state="visible" r:id="rId499"/>
-    <sheet name="LegalMeasure" sheetId="500" state="visible" r:id="rId500"/>
-    <sheet name="LegalObligation" sheetId="501" state="visible" r:id="rId501"/>
-    <sheet name="LegalObligationCompleted" sheetId="502" state="visible" r:id="rId502"/>
-    <sheet name="LegalObligationOngoing" sheetId="503" state="visible" r:id="rId503"/>
-    <sheet name="LegalObligationPending" sheetId="504" state="visible" r:id="rId504"/>
-    <sheet name="LegalObligationStatus" sheetId="505" state="visible" r:id="rId505"/>
-    <sheet name="LegitimateInterest" sheetId="506" state="visible" r:id="rId506"/>
-    <sheet name="LegitimateInterestAssessment" sheetId="507" state="visible" r:id="rId507"/>
-    <sheet name="LegitimateInterestInformed" sheetId="508" state="visible" r:id="rId508"/>
-    <sheet name="LegitimateInterestNotObjected" sheetId="509" state="visible" r:id="rId509"/>
-    <sheet name="LegitimateInterestObjected" sheetId="510" state="visible" r:id="rId510"/>
-    <sheet name="LegitimateInterestOfController" sheetId="511" state="visible" r:id="rId511"/>
-    <sheet name="LegitimateInterestOfDataSubject" sheetId="512" state="visible" r:id="rId512"/>
-    <sheet name="LegitimateInterestOfThirdParty" sheetId="513" state="visible" r:id="rId513"/>
-    <sheet name="LegitimateInterestStatus" sheetId="514" state="visible" r:id="rId514"/>
-    <sheet name="LegitimateInterestUninformed" sheetId="515" state="visible" r:id="rId515"/>
-    <sheet name="LicenseAgreement" sheetId="516" state="visible" r:id="rId516"/>
-    <sheet name="Likelihood" sheetId="517" state="visible" r:id="rId517"/>
-    <sheet name="LocalEnvironmentScale" sheetId="518" state="visible" r:id="rId518"/>
-    <sheet name="LocalLocation" sheetId="519" state="visible" r:id="rId519"/>
-    <sheet name="LocalityScale" sheetId="520" state="visible" r:id="rId520"/>
-    <sheet name="LocationFixture" sheetId="521" state="visible" r:id="rId521"/>
-    <sheet name="LocationLocality" sheetId="522" state="visible" r:id="rId522"/>
-    <sheet name="LoggingPolicy" sheetId="523" state="visible" r:id="rId523"/>
-    <sheet name="MaintainFraudDatabase" sheetId="524" state="visible" r:id="rId524"/>
-    <sheet name="MakeAvailable" sheetId="525" state="visible" r:id="rId525"/>
-    <sheet name="ManageConsent" sheetId="526" state="visible" r:id="rId526"/>
-    <sheet name="ManagementStandard" sheetId="527" state="visible" r:id="rId527"/>
-    <sheet name="Marketing" sheetId="528" state="visible" r:id="rId528"/>
-    <sheet name="Match" sheetId="529" state="visible" r:id="rId529"/>
-    <sheet name="MediumDataVolume" sheetId="530" state="visible" r:id="rId530"/>
-    <sheet name="MediumScaleOfDataSubjects" sheetId="531" state="visible" r:id="rId531"/>
-    <sheet name="MediumScaleProcessing" sheetId="532" state="visible" r:id="rId532"/>
-    <sheet name="Member" sheetId="533" state="visible" r:id="rId533"/>
-    <sheet name="MemberPartnerManagement" sheetId="534" state="visible" r:id="rId534"/>
-    <sheet name="MentallyVulnerableDataSubject" sheetId="535" state="visible" r:id="rId535"/>
-    <sheet name="MentallyVulnerableHuman" sheetId="536" state="visible" r:id="rId536"/>
-    <sheet name="MessageAuthenticationCodes" sheetId="537" state="visible" r:id="rId537"/>
-    <sheet name="MetadataManagement" sheetId="538" state="visible" r:id="rId538"/>
-    <sheet name="MisusePreventionAndDetection" sheetId="539" state="visible" r:id="rId539"/>
-    <sheet name="MobilePlatformSecurity" sheetId="540" state="visible" r:id="rId540"/>
-    <sheet name="Modify" sheetId="541" state="visible" r:id="rId541"/>
-    <sheet name="Monitor" sheetId="542" state="visible" r:id="rId542"/>
-    <sheet name="MonitoringPolicy" sheetId="543" state="visible" r:id="rId543"/>
-    <sheet name="MonotonicCounterPseudonymisation" sheetId="544" state="visible" r:id="rId544"/>
-    <sheet name="Move" sheetId="545" state="visible" r:id="rId545"/>
-    <sheet name="MultiFactorAuthentication" sheetId="546" state="visible" r:id="rId546"/>
-    <sheet name="MultiNationalScale" sheetId="547" state="visible" r:id="rId547"/>
-    <sheet name="NDA" sheetId="548" state="visible" r:id="rId548"/>
-    <sheet name="NationalAuthority" sheetId="549" state="visible" r:id="rId549"/>
-    <sheet name="NationalScale" sheetId="550" state="visible" r:id="rId550"/>
-    <sheet name="NaturalPerson" sheetId="551" state="visible" r:id="rId551"/>
-    <sheet name="NearlyGlobalScale" sheetId="552" state="visible" r:id="rId552"/>
-    <sheet name="Necessity" sheetId="553" state="visible" r:id="rId553"/>
-    <sheet name="NegotiateContract" sheetId="554" state="visible" r:id="rId554"/>
-    <sheet name="NegotiatedContract" sheetId="555" state="visible" r:id="rId555"/>
-    <sheet name="NetworkProxyRouting" sheetId="556" state="visible" r:id="rId556"/>
-    <sheet name="NetworkSecurityProtocols" sheetId="557" state="visible" r:id="rId557"/>
-    <sheet name="NonCitizen" sheetId="558" state="visible" r:id="rId558"/>
-    <sheet name="NonCommercialPurpose" sheetId="559" state="visible" r:id="rId559"/>
-    <sheet name="NonCommercialResearch" sheetId="560" state="visible" r:id="rId560"/>
-    <sheet name="NonCompliant" sheetId="561" state="visible" r:id="rId561"/>
-    <sheet name="NonConformant" sheetId="562" state="visible" r:id="rId562"/>
-    <sheet name="NonGovernmentalOrganisation" sheetId="563" state="visible" r:id="rId563"/>
-    <sheet name="NonPersonalData" sheetId="564" state="visible" r:id="rId564"/>
-    <sheet name="NonPersonalDataProcess" sheetId="565" state="visible" r:id="rId565"/>
-    <sheet name="NonProfitOrganisation" sheetId="566" state="visible" r:id="rId566"/>
-    <sheet name="NonPublicDataSource" sheetId="567" state="visible" r:id="rId567"/>
-    <sheet name="NotApplicable" sheetId="568" state="visible" r:id="rId568"/>
-    <sheet name="NotAutomated" sheetId="569" state="visible" r:id="rId569"/>
-    <sheet name="NotAvailable" sheetId="570" state="visible" r:id="rId570"/>
-    <sheet name="NotInvolved" sheetId="571" state="visible" r:id="rId571"/>
-    <sheet name="NotRequired" sheetId="572" state="visible" r:id="rId572"/>
-    <sheet name="Notice" sheetId="573" state="visible" r:id="rId573"/>
-    <sheet name="NoticeCommunicated" sheetId="574" state="visible" r:id="rId574"/>
-    <sheet name="NoticeGenerated" sheetId="575" state="visible" r:id="rId575"/>
-    <sheet name="NoticeIcon" sheetId="576" state="visible" r:id="rId576"/>
-    <sheet name="NoticeLatest" sheetId="577" state="visible" r:id="rId577"/>
-    <sheet name="NoticeLayer" sheetId="578" state="visible" r:id="rId578"/>
-    <sheet name="NoticeStale" sheetId="579" state="visible" r:id="rId579"/>
-    <sheet name="NoticeStatus" sheetId="580" state="visible" r:id="rId580"/>
-    <sheet name="NoticeUnused" sheetId="581" state="visible" r:id="rId581"/>
-    <sheet name="NoticeUpdated" sheetId="582" state="visible" r:id="rId582"/>
-    <sheet name="NoticeUsed" sheetId="583" state="visible" r:id="rId583"/>
-    <sheet name="Notification" sheetId="584" state="visible" r:id="rId584"/>
-    <sheet name="NotificationCompleted" sheetId="585" state="visible" r:id="rId585"/>
-    <sheet name="NotificationFailed" sheetId="586" state="visible" r:id="rId586"/>
-    <sheet name="NotificationNotNeeded" sheetId="587" state="visible" r:id="rId587"/>
-    <sheet name="NotificationOngoing" sheetId="588" state="visible" r:id="rId588"/>
-    <sheet name="NotificationPlanned" sheetId="589" state="visible" r:id="rId589"/>
-    <sheet name="NotificationStatus" sheetId="590" state="visible" r:id="rId590"/>
-    <sheet name="ObjectingToProcess" sheetId="591" state="visible" r:id="rId591"/>
-    <sheet name="Obligation" sheetId="592" state="visible" r:id="rId592"/>
-    <sheet name="ObligationFulfilled" sheetId="593" state="visible" r:id="rId593"/>
-    <sheet name="ObligationUnfulfilled" sheetId="594" state="visible" r:id="rId594"/>
-    <sheet name="ObligationViolated" sheetId="595" state="visible" r:id="rId595"/>
-    <sheet name="Observe" sheetId="596" state="visible" r:id="rId596"/>
-    <sheet name="ObservedData" sheetId="597" state="visible" r:id="rId597"/>
-    <sheet name="ObservedPersonalData" sheetId="598" state="visible" r:id="rId598"/>
-    <sheet name="Obtain" sheetId="599" state="visible" r:id="rId599"/>
-    <sheet name="ObtainConsent" sheetId="600" state="visible" r:id="rId600"/>
-    <sheet name="OfferContract" sheetId="601" state="visible" r:id="rId601"/>
-    <sheet name="OfficialAuthorityExerciseCompleted" sheetId="602" state="visible" r:id="rId602"/>
-    <sheet name="OfficialAuthorityExerciseOngoing" sheetId="603" state="visible" r:id="rId603"/>
-    <sheet name="OfficialAuthorityExercisePending" sheetId="604" state="visible" r:id="rId604"/>
-    <sheet name="OfficialAuthorityExerciseStatus" sheetId="605" state="visible" r:id="rId605"/>
-    <sheet name="OfficialAuthorityOfController" sheetId="606" state="visible" r:id="rId606"/>
-    <sheet name="OftenFrequency" sheetId="607" state="visible" r:id="rId607"/>
-    <sheet name="OperatingSystemSecurity" sheetId="608" state="visible" r:id="rId608"/>
-    <sheet name="OptimisationForConsumer" sheetId="609" state="visible" r:id="rId609"/>
-    <sheet name="OptimisationForController" sheetId="610" state="visible" r:id="rId610"/>
-    <sheet name="OptimiseUserInterface" sheetId="611" state="visible" r:id="rId611"/>
-    <sheet name="OptingInToProcess" sheetId="612" state="visible" r:id="rId612"/>
-    <sheet name="OptingOutFromProcess" sheetId="613" state="visible" r:id="rId613"/>
-    <sheet name="OralNotice" sheetId="614" state="visible" r:id="rId614"/>
-    <sheet name="OrganisationComplianceManagement" sheetId="615" state="visible" r:id="rId615"/>
-    <sheet name="OrganisationGovernance" sheetId="616" state="visible" r:id="rId616"/>
-    <sheet name="OrganisationRiskManagement" sheetId="617" state="visible" r:id="rId617"/>
-    <sheet name="OrganisationalMeasure" sheetId="618" state="visible" r:id="rId618"/>
-    <sheet name="OrganisationalUnit" sheetId="619" state="visible" r:id="rId619"/>
-    <sheet name="Organise" sheetId="620" state="visible" r:id="rId620"/>
-    <sheet name="PIA" sheetId="621" state="visible" r:id="rId621"/>
-    <sheet name="ParentLegalEntity" sheetId="622" state="visible" r:id="rId622"/>
-    <sheet name="ParentOfDataSubject" sheetId="623" state="visible" r:id="rId623"/>
-    <sheet name="ParentOfHuman" sheetId="624" state="visible" r:id="rId624"/>
-    <sheet name="PartialAutomation" sheetId="625" state="visible" r:id="rId625"/>
-    <sheet name="PartiallyCompliant" sheetId="626" state="visible" r:id="rId626"/>
-    <sheet name="Participant" sheetId="627" state="visible" r:id="rId627"/>
-    <sheet name="PassiveRight" sheetId="628" state="visible" r:id="rId628"/>
-    <sheet name="PassivelyInvolved" sheetId="629" state="visible" r:id="rId629"/>
-    <sheet name="PasswordAuthentication" sheetId="630" state="visible" r:id="rId630"/>
-    <sheet name="Patient" sheetId="631" state="visible" r:id="rId631"/>
-    <sheet name="PaymentManagement" sheetId="632" state="visible" r:id="rId632"/>
-    <sheet name="PenetrationTestingMethods" sheetId="633" state="visible" r:id="rId633"/>
-    <sheet name="Permission" sheetId="634" state="visible" r:id="rId634"/>
-    <sheet name="PermissionManagement" sheetId="635" state="visible" r:id="rId635"/>
-    <sheet name="PermissionNotUtilised" sheetId="636" state="visible" r:id="rId636"/>
-    <sheet name="PermissionUtilised" sheetId="637" state="visible" r:id="rId637"/>
-    <sheet name="PersonalData" sheetId="638" state="visible" r:id="rId638"/>
-    <sheet name="PersonalDataAudit" sheetId="639" state="visible" r:id="rId639"/>
-    <sheet name="PersonalDataHandling" sheetId="640" state="visible" r:id="rId640"/>
-    <sheet name="PersonalDataProcess" sheetId="641" state="visible" r:id="rId641"/>
-    <sheet name="PersonalSpace" sheetId="642" state="visible" r:id="rId642"/>
-    <sheet name="Personalisation" sheetId="643" state="visible" r:id="rId643"/>
-    <sheet name="PersonalisedAdvertising" sheetId="644" state="visible" r:id="rId644"/>
-    <sheet name="PersonalisedBenefits" sheetId="645" state="visible" r:id="rId645"/>
-    <sheet name="PersonnelBehaviourMonitoring" sheetId="646" state="visible" r:id="rId646"/>
-    <sheet name="PersonnelHiring" sheetId="647" state="visible" r:id="rId647"/>
-    <sheet name="PersonnelManagement" sheetId="648" state="visible" r:id="rId648"/>
-    <sheet name="PersonnelMonitoring" sheetId="649" state="visible" r:id="rId649"/>
-    <sheet name="PersonnelOffboarding" sheetId="650" state="visible" r:id="rId650"/>
-    <sheet name="PersonnelOnboarding" sheetId="651" state="visible" r:id="rId651"/>
-    <sheet name="PersonnelPayment" sheetId="652" state="visible" r:id="rId652"/>
-    <sheet name="PersonnelPerformanceEvaluation" sheetId="653" state="visible" r:id="rId653"/>
-    <sheet name="PersonnelPerformanceManagement" sheetId="654" state="visible" r:id="rId654"/>
-    <sheet name="PersonnelPerformanceMonitoring" sheetId="655" state="visible" r:id="rId655"/>
-    <sheet name="PersonnelPerformancePrediction" sheetId="656" state="visible" r:id="rId656"/>
-    <sheet name="PersonnelPromotionManagement" sheetId="657" state="visible" r:id="rId657"/>
-    <sheet name="PersonnelTerminationManagement" sheetId="658" state="visible" r:id="rId658"/>
-    <sheet name="PersonnelWorkloadManagement" sheetId="659" state="visible" r:id="rId659"/>
-    <sheet name="PhysicalAccessControlMethod" sheetId="660" state="visible" r:id="rId660"/>
-    <sheet name="PhysicalAuthentication" sheetId="661" state="visible" r:id="rId661"/>
-    <sheet name="PhysicalAuthorisation" sheetId="662" state="visible" r:id="rId662"/>
-    <sheet name="PhysicalDeviceSecurity" sheetId="663" state="visible" r:id="rId663"/>
-    <sheet name="PhysicalInterceptionProtection" sheetId="664" state="visible" r:id="rId664"/>
-    <sheet name="PhysicalInterruptionProtection" sheetId="665" state="visible" r:id="rId665"/>
-    <sheet name="PhysicalMeasure" sheetId="666" state="visible" r:id="rId666"/>
-    <sheet name="PhysicalNetworkSecurity" sheetId="667" state="visible" r:id="rId667"/>
-    <sheet name="PhysicalSecureStorage" sheetId="668" state="visible" r:id="rId668"/>
-    <sheet name="PhysicalSupplySecurity" sheetId="669" state="visible" r:id="rId669"/>
-    <sheet name="PhysicalSurveillance" sheetId="670" state="visible" r:id="rId670"/>
-    <sheet name="Policy" sheetId="671" state="visible" r:id="rId671"/>
-    <sheet name="PoliticalCampaign" sheetId="672" state="visible" r:id="rId672"/>
-    <sheet name="PostQuantumCryptography" sheetId="673" state="visible" r:id="rId673"/>
-    <sheet name="PostedNotice" sheetId="674" state="visible" r:id="rId674"/>
-    <sheet name="PrimaryImportance" sheetId="675" state="visible" r:id="rId675"/>
-    <sheet name="PrimaryUse" sheetId="676" state="visible" r:id="rId676"/>
-    <sheet name="Principle" sheetId="677" state="visible" r:id="rId677"/>
-    <sheet name="PrintedNotice" sheetId="678" state="visible" r:id="rId678"/>
-    <sheet name="PrivacyByDefault" sheetId="679" state="visible" r:id="rId679"/>
-    <sheet name="PrivacyByDesign" sheetId="680" state="visible" r:id="rId680"/>
-    <sheet name="PrivacyNotice" sheetId="681" state="visible" r:id="rId681"/>
-    <sheet name="PrivacyPreservingProtocol" sheetId="682" state="visible" r:id="rId682"/>
-    <sheet name="PrivateCommunalSpace" sheetId="683" state="visible" r:id="rId683"/>
-    <sheet name="PrivateInformationRetrieval" sheetId="684" state="visible" r:id="rId684"/>
-    <sheet name="PrivateLocation" sheetId="685" state="visible" r:id="rId685"/>
-    <sheet name="PrivateSectorBody" sheetId="686" state="visible" r:id="rId686"/>
-    <sheet name="PrivateSpace" sheetId="687" state="visible" r:id="rId687"/>
-    <sheet name="PrivatelyOperatedPublicSpace" sheetId="688" state="visible" r:id="rId688"/>
-    <sheet name="PrivatelyOwnedPublicSpace" sheetId="689" state="visible" r:id="rId689"/>
-    <sheet name="PrivatelyOwnedSpace" sheetId="690" state="visible" r:id="rId690"/>
-    <sheet name="Processing" sheetId="691" state="visible" r:id="rId691"/>
-    <sheet name="ProcessingCondition" sheetId="692" state="visible" r:id="rId692"/>
-    <sheet name="ProcessingContext" sheetId="693" state="visible" r:id="rId693"/>
-    <sheet name="ProcessingDuration" sheetId="694" state="visible" r:id="rId694"/>
-    <sheet name="ProcessingLocation" sheetId="695" state="visible" r:id="rId695"/>
-    <sheet name="ProcessingScale" sheetId="696" state="visible" r:id="rId696"/>
-    <sheet name="ProfessionalConfidentialData" sheetId="697" state="visible" r:id="rId697"/>
-    <sheet name="ProfessionalTraining" sheetId="698" state="visible" r:id="rId698"/>
-    <sheet name="Profiling" sheetId="699" state="visible" r:id="rId699"/>
-    <sheet name="Prohibition" sheetId="700" state="visible" r:id="rId700"/>
-    <sheet name="ProhibitionUnviolated" sheetId="701" state="visible" r:id="rId701"/>
-    <sheet name="ProhibitionViolated" sheetId="702" state="visible" r:id="rId702"/>
-    <sheet name="ProtectionOfIPR" sheetId="703" state="visible" r:id="rId703"/>
-    <sheet name="ProtectionOfNationalSecurity" sheetId="704" state="visible" r:id="rId704"/>
-    <sheet name="ProtectionOfPublicSecurity" sheetId="705" state="visible" r:id="rId705"/>
-    <sheet name="ProvideConsent" sheetId="706" state="visible" r:id="rId706"/>
-    <sheet name="ProvideEventRecommendations" sheetId="707" state="visible" r:id="rId707"/>
-    <sheet name="ProvideOfficialStatistics" sheetId="708" state="visible" r:id="rId708"/>
-    <sheet name="ProvidePersonalisedRecommendations" sheetId="709" state="visible" r:id="rId709"/>
-    <sheet name="ProvideProductRecommendations" sheetId="710" state="visible" r:id="rId710"/>
-    <sheet name="ProvidedData" sheetId="711" state="visible" r:id="rId711"/>
-    <sheet name="ProvidedPersonalData" sheetId="712" state="visible" r:id="rId712"/>
-    <sheet name="ProviderStandardFormContract" sheetId="713" state="visible" r:id="rId713"/>
-    <sheet name="Pseudonymisation" sheetId="714" state="visible" r:id="rId714"/>
-    <sheet name="Pseudonymise" sheetId="715" state="visible" r:id="rId715"/>
-    <sheet name="PseudonymisedData" sheetId="716" state="visible" r:id="rId716"/>
-    <sheet name="PublicBenefit" sheetId="717" state="visible" r:id="rId717"/>
-    <sheet name="PublicDataSource" sheetId="718" state="visible" r:id="rId718"/>
-    <sheet name="PublicInterest" sheetId="719" state="visible" r:id="rId719"/>
-    <sheet name="PublicInterestCompleted" sheetId="720" state="visible" r:id="rId720"/>
-    <sheet name="PublicInterestObjected" sheetId="721" state="visible" r:id="rId721"/>
-    <sheet name="PublicInterestOngoing" sheetId="722" state="visible" r:id="rId722"/>
-    <sheet name="PublicInterestPending" sheetId="723" state="visible" r:id="rId723"/>
-    <sheet name="PublicInterestStatus" sheetId="724" state="visible" r:id="rId724"/>
-    <sheet name="PublicLocation" sheetId="725" state="visible" r:id="rId725"/>
-    <sheet name="PublicPolicyMaking" sheetId="726" state="visible" r:id="rId726"/>
-    <sheet name="PublicRegisterOfEntities" sheetId="727" state="visible" r:id="rId727"/>
-    <sheet name="PublicRelations" sheetId="728" state="visible" r:id="rId728"/>
-    <sheet name="PublicSectorBody" sheetId="729" state="visible" r:id="rId729"/>
-    <sheet name="PublicSpace" sheetId="730" state="visible" r:id="rId730"/>
-    <sheet name="PubliclyAccessibleSpace" sheetId="731" state="visible" r:id="rId731"/>
-    <sheet name="PubliclyOwnedSpace" sheetId="732" state="visible" r:id="rId732"/>
-    <sheet name="Purpose" sheetId="733" state="visible" r:id="rId733"/>
-    <sheet name="QuantumCryptography" sheetId="734" state="visible" r:id="rId734"/>
-    <sheet name="Query" sheetId="735" state="visible" r:id="rId735"/>
-    <sheet name="RNGPseudonymisation" sheetId="736" state="visible" r:id="rId736"/>
-    <sheet name="ROPA" sheetId="737" state="visible" r:id="rId737"/>
-    <sheet name="RandomLocation" sheetId="738" state="visible" r:id="rId738"/>
-    <sheet name="ReaffirmConsent" sheetId="739" state="visible" r:id="rId739"/>
-    <sheet name="RecertificationPolicy" sheetId="740" state="visible" r:id="rId740"/>
-    <sheet name="RecipientInformed" sheetId="741" state="visible" r:id="rId741"/>
-    <sheet name="RecipientUninformed" sheetId="742" state="visible" r:id="rId742"/>
-    <sheet name="Recommendation" sheetId="743" state="visible" r:id="rId743"/>
-    <sheet name="RecommendationFollowed" sheetId="744" state="visible" r:id="rId744"/>
-    <sheet name="RecommendationNotFollowed" sheetId="745" state="visible" r:id="rId745"/>
-    <sheet name="RecordManagement" sheetId="746" state="visible" r:id="rId746"/>
-    <sheet name="RecordsOfActivities" sheetId="747" state="visible" r:id="rId747"/>
-    <sheet name="RecruitmentAdvertising" sheetId="748" state="visible" r:id="rId748"/>
-    <sheet name="RecruitmentApplicantBackgroundCheck" sheetId="749" state="visible" r:id="rId749"/>
-    <sheet name="RecruitmentApplicantCriminalBackgroundCheck" sheetId="750" state="visible" r:id="rId750"/>
-    <sheet name="RecruitmentApplicantInformationAuthentication" sheetId="751" state="visible" r:id="rId751"/>
-    <sheet name="RecruitmentApplicantSelection" sheetId="752" state="visible" r:id="rId752"/>
-    <sheet name="RecruitmentApplicationAnalysis" sheetId="753" state="visible" r:id="rId753"/>
-    <sheet name="RecruitmentApplicationManagement" sheetId="754" state="visible" r:id="rId754"/>
-    <sheet name="RecruitmentApplicationScreening" sheetId="755" state="visible" r:id="rId755"/>
-    <sheet name="RecruitmentInterviewAnalysis" sheetId="756" state="visible" r:id="rId756"/>
-    <sheet name="RecruitmentInterviewAssessment" sheetId="757" state="visible" r:id="rId757"/>
-    <sheet name="RecruitmentInterviewManagement" sheetId="758" state="visible" r:id="rId758"/>
-    <sheet name="RecruitmentInterviewScheduling" sheetId="759" state="visible" r:id="rId759"/>
-    <sheet name="RecruitmentManagement" sheetId="760" state="visible" r:id="rId760"/>
-    <sheet name="RecruitmentTargetedAdvertising" sheetId="761" state="visible" r:id="rId761"/>
-    <sheet name="Reformat" sheetId="762" state="visible" r:id="rId762"/>
-    <sheet name="RefuseConsent" sheetId="763" state="visible" r:id="rId763"/>
-    <sheet name="RefuseContract" sheetId="764" state="visible" r:id="rId764"/>
-    <sheet name="RegionalAuthority" sheetId="765" state="visible" r:id="rId765"/>
-    <sheet name="RegionalScale" sheetId="766" state="visible" r:id="rId766"/>
-    <sheet name="RegulatorySandbox" sheetId="767" state="visible" r:id="rId767"/>
-    <sheet name="ReligiousAssociations" sheetId="768" state="visible" r:id="rId768"/>
-    <sheet name="RemoteLocation" sheetId="769" state="visible" r:id="rId769"/>
-    <sheet name="Remove" sheetId="770" state="visible" r:id="rId770"/>
-    <sheet name="RenewedConsentGiven" sheetId="771" state="visible" r:id="rId771"/>
-    <sheet name="RepairImpairments" sheetId="772" state="visible" r:id="rId772"/>
-    <sheet name="Representative" sheetId="773" state="visible" r:id="rId773"/>
-    <sheet name="RequestAccepted" sheetId="774" state="visible" r:id="rId774"/>
-    <sheet name="RequestAcknowledged" sheetId="775" state="visible" r:id="rId775"/>
-    <sheet name="RequestActionDelayed" sheetId="776" state="visible" r:id="rId776"/>
-    <sheet name="RequestFulfilled" sheetId="777" state="visible" r:id="rId777"/>
-    <sheet name="RequestInitiated" sheetId="778" state="visible" r:id="rId778"/>
-    <sheet name="RequestRejected" sheetId="779" state="visible" r:id="rId779"/>
-    <sheet name="RequestRequiredActionPerformed" sheetId="780" state="visible" r:id="rId780"/>
-    <sheet name="RequestRequiresAction" sheetId="781" state="visible" r:id="rId781"/>
-    <sheet name="RequestStatus" sheetId="782" state="visible" r:id="rId782"/>
-    <sheet name="RequestStatusQuery" sheetId="783" state="visible" r:id="rId783"/>
-    <sheet name="RequestUnfulfilled" sheetId="784" state="visible" r:id="rId784"/>
-    <sheet name="RequestedServiceProvision" sheetId="785" state="visible" r:id="rId785"/>
-    <sheet name="Required" sheetId="786" state="visible" r:id="rId786"/>
-    <sheet name="ResearchAndDevelopment" sheetId="787" state="visible" r:id="rId787"/>
-    <sheet name="ResidualRisk" sheetId="788" state="visible" r:id="rId788"/>
-    <sheet name="Restrict" sheetId="789" state="visible" r:id="rId789"/>
-    <sheet name="Retrieve" sheetId="790" state="visible" r:id="rId790"/>
-    <sheet name="ReuseCompatibility" sheetId="791" state="visible" r:id="rId791"/>
-    <sheet name="ReversingProcessEffects" sheetId="792" state="visible" r:id="rId792"/>
-    <sheet name="ReversingProcessInput" sheetId="793" state="visible" r:id="rId793"/>
-    <sheet name="ReversingProcessOutput" sheetId="794" state="visible" r:id="rId794"/>
-    <sheet name="ReviewImpactAssessment" sheetId="795" state="visible" r:id="rId795"/>
-    <sheet name="ReviewProcedure" sheetId="796" state="visible" r:id="rId796"/>
-    <sheet name="Right" sheetId="797" state="visible" r:id="rId797"/>
-    <sheet name="RightExerciseActivity" sheetId="798" state="visible" r:id="rId798"/>
-    <sheet name="RightExerciseNotice" sheetId="799" state="visible" r:id="rId799"/>
-    <sheet name="RightExerciseRecord" sheetId="800" state="visible" r:id="rId800"/>
-    <sheet name="RightFulfilmentNotice" sheetId="801" state="visible" r:id="rId801"/>
-    <sheet name="RightNonFulfilmentNotice" sheetId="802" state="visible" r:id="rId802"/>
-    <sheet name="RightNotice" sheetId="803" state="visible" r:id="rId803"/>
-    <sheet name="RightsFulfilment" sheetId="804" state="visible" r:id="rId804"/>
-    <sheet name="RightsImpactAssessment" sheetId="805" state="visible" r:id="rId805"/>
-    <sheet name="RightsManagement" sheetId="806" state="visible" r:id="rId806"/>
-    <sheet name="Risk" sheetId="807" state="visible" r:id="rId807"/>
-    <sheet name="RiskAssessment" sheetId="808" state="visible" r:id="rId808"/>
-    <sheet name="RiskConcept" sheetId="809" state="visible" r:id="rId809"/>
-    <sheet name="RiskLevel" sheetId="810" state="visible" r:id="rId810"/>
-    <sheet name="RiskMitigationMeasure" sheetId="811" state="visible" r:id="rId811"/>
-    <sheet name="Rule" sheetId="812" state="visible" r:id="rId812"/>
-    <sheet name="RuleFulfilled" sheetId="813" state="visible" r:id="rId813"/>
-    <sheet name="RuleFulfilmentStatus" sheetId="814" state="visible" r:id="rId814"/>
-    <sheet name="RuleUnfulfilled" sheetId="815" state="visible" r:id="rId815"/>
-    <sheet name="RuleViolated" sheetId="816" state="visible" r:id="rId816"/>
-    <sheet name="SMEOrganisation" sheetId="817" state="visible" r:id="rId817"/>
-    <sheet name="Safeguard" sheetId="818" state="visible" r:id="rId818"/>
-    <sheet name="SafeguardForDataTransfer" sheetId="819" state="visible" r:id="rId819"/>
-    <sheet name="Scale" sheetId="820" state="visible" r:id="rId820"/>
-    <sheet name="ScientificResearch" sheetId="821" state="visible" r:id="rId821"/>
-    <sheet name="Scope" sheetId="822" state="visible" r:id="rId822"/>
-    <sheet name="ScoringOfIndividuals" sheetId="823" state="visible" r:id="rId823"/>
-    <sheet name="Screen" sheetId="824" state="visible" r:id="rId824"/>
-    <sheet name="Seal" sheetId="825" state="visible" r:id="rId825"/>
-    <sheet name="SearchFunctionalities" sheetId="826" state="visible" r:id="rId826"/>
-    <sheet name="SecondaryImportance" sheetId="827" state="visible" r:id="rId827"/>
-    <sheet name="SecondaryUse" sheetId="828" state="visible" r:id="rId828"/>
-    <sheet name="SecretSharingSchemes" sheetId="829" state="visible" r:id="rId829"/>
-    <sheet name="Sector" sheetId="830" state="visible" r:id="rId830"/>
-    <sheet name="SecureMultiPartyComputation" sheetId="831" state="visible" r:id="rId831"/>
-    <sheet name="SecureProcessingEnvironment" sheetId="832" state="visible" r:id="rId832"/>
-    <sheet name="SecurityAssessment" sheetId="833" state="visible" r:id="rId833"/>
-    <sheet name="SecurityAudit" sheetId="834" state="visible" r:id="rId834"/>
-    <sheet name="SecurityIncidentNotice" sheetId="835" state="visible" r:id="rId835"/>
-    <sheet name="SecurityIncidentNotification" sheetId="836" state="visible" r:id="rId836"/>
-    <sheet name="SecurityIncidentRecord" sheetId="837" state="visible" r:id="rId837"/>
-    <sheet name="SecurityKnowledgeTraining" sheetId="838" state="visible" r:id="rId838"/>
-    <sheet name="SecurityMethod" sheetId="839" state="visible" r:id="rId839"/>
-    <sheet name="SecurityProcedure" sheetId="840" state="visible" r:id="rId840"/>
-    <sheet name="SecurityRoleProcedures" sheetId="841" state="visible" r:id="rId841"/>
-    <sheet name="SellDataToThirdParties" sheetId="842" state="visible" r:id="rId842"/>
-    <sheet name="SellInsightsFromData" sheetId="843" state="visible" r:id="rId843"/>
-    <sheet name="SellProducts" sheetId="844" state="visible" r:id="rId844"/>
-    <sheet name="SellProductsToDataSubject" sheetId="845" state="visible" r:id="rId845"/>
-    <sheet name="SemiPrivateSpace" sheetId="846" state="visible" r:id="rId846"/>
-    <sheet name="SensitiveData" sheetId="847" state="visible" r:id="rId847"/>
-    <sheet name="SensitiveNonPersonalData" sheetId="848" state="visible" r:id="rId848"/>
-    <sheet name="SensitivePersonalData" sheetId="849" state="visible" r:id="rId849"/>
-    <sheet name="SensitivityLevel" sheetId="850" state="visible" r:id="rId850"/>
-    <sheet name="ServiceAccessDetermination" sheetId="851" state="visible" r:id="rId851"/>
-    <sheet name="ServiceConsumer" sheetId="852" state="visible" r:id="rId852"/>
-    <sheet name="ServiceLevelAgreement" sheetId="853" state="visible" r:id="rId853"/>
-    <sheet name="ServiceManagement" sheetId="854" state="visible" r:id="rId854"/>
-    <sheet name="ServiceMonitoring" sheetId="855" state="visible" r:id="rId855"/>
-    <sheet name="ServiceOptimisation" sheetId="856" state="visible" r:id="rId856"/>
-    <sheet name="ServicePersonalisation" sheetId="857" state="visible" r:id="rId857"/>
-    <sheet name="ServiceProvider" sheetId="858" state="visible" r:id="rId858"/>
-    <sheet name="ServiceProvision" sheetId="859" state="visible" r:id="rId859"/>
-    <sheet name="ServiceRegistration" sheetId="860" state="visible" r:id="rId860"/>
-    <sheet name="ServiceUsageAnalytics" sheetId="861" state="visible" r:id="rId861"/>
-    <sheet name="Severity" sheetId="862" state="visible" r:id="rId862"/>
-    <sheet name="Share" sheetId="863" state="visible" r:id="rId863"/>
-    <sheet name="SingleSignOn" sheetId="864" state="visible" r:id="rId864"/>
-    <sheet name="SingularDataVolume" sheetId="865" state="visible" r:id="rId865"/>
-    <sheet name="SingularFrequency" sheetId="866" state="visible" r:id="rId866"/>
-    <sheet name="SingularScaleOfDataSubjects" sheetId="867" state="visible" r:id="rId867"/>
-    <sheet name="SmallDataVolume" sheetId="868" state="visible" r:id="rId868"/>
-    <sheet name="SmallScaleOfDataSubjects" sheetId="869" state="visible" r:id="rId869"/>
-    <sheet name="SmallScaleProcessing" sheetId="870" state="visible" r:id="rId870"/>
-    <sheet name="SocialMediaMarketing" sheetId="871" state="visible" r:id="rId871"/>
-    <sheet name="SpecialCategoryPersonalData" sheetId="872" state="visible" r:id="rId872"/>
-    <sheet name="SporadicDataVolume" sheetId="873" state="visible" r:id="rId873"/>
-    <sheet name="SporadicFrequency" sheetId="874" state="visible" r:id="rId874"/>
-    <sheet name="SporadicScaleOfDataSubjects" sheetId="875" state="visible" r:id="rId875"/>
-    <sheet name="StaffTraining" sheetId="876" state="visible" r:id="rId876"/>
-    <sheet name="Standard" sheetId="877" state="visible" r:id="rId877"/>
-    <sheet name="StandardFormContract" sheetId="878" state="visible" r:id="rId878"/>
-    <sheet name="StandardsConformance" sheetId="879" state="visible" r:id="rId879"/>
-    <sheet name="StartupOrganisation" sheetId="880" state="visible" r:id="rId880"/>
-    <sheet name="StatisticalConfidentialityAgreement" sheetId="881" state="visible" r:id="rId881"/>
-    <sheet name="StatisticallyConfidentialData" sheetId="882" state="visible" r:id="rId882"/>
-    <sheet name="Status" sheetId="883" state="visible" r:id="rId883"/>
-    <sheet name="StorageCondition" sheetId="884" state="visible" r:id="rId884"/>
-    <sheet name="StorageDeletion" sheetId="885" state="visible" r:id="rId885"/>
-    <sheet name="StorageDuration" sheetId="886" state="visible" r:id="rId886"/>
-    <sheet name="StorageLocation" sheetId="887" state="visible" r:id="rId887"/>
-    <sheet name="StorageRestoration" sheetId="888" state="visible" r:id="rId888"/>
-    <sheet name="Store" sheetId="889" state="visible" r:id="rId889"/>
-    <sheet name="Structure" sheetId="890" state="visible" r:id="rId890"/>
-    <sheet name="Student" sheetId="891" state="visible" r:id="rId891"/>
-    <sheet name="SubProcessorAgreement" sheetId="892" state="visible" r:id="rId892"/>
-    <sheet name="Subscriber" sheetId="893" state="visible" r:id="rId893"/>
-    <sheet name="SubsidiaryLegalEntity" sheetId="894" state="visible" r:id="rId894"/>
-    <sheet name="SupportContractNegotiation" sheetId="895" state="visible" r:id="rId895"/>
-    <sheet name="SupportEntityDecisionMaking" sheetId="896" state="visible" r:id="rId896"/>
-    <sheet name="SupportExchangeOfViews" sheetId="897" state="visible" r:id="rId897"/>
-    <sheet name="SupportInformedConsentDecision" sheetId="898" state="visible" r:id="rId898"/>
-    <sheet name="SupraNationalAuthority" sheetId="899" state="visible" r:id="rId899"/>
-    <sheet name="SupraNationalUnion" sheetId="900" state="visible" r:id="rId900"/>
-    <sheet name="SymmetricCryptography" sheetId="901" state="visible" r:id="rId901"/>
-    <sheet name="SymmetricEncryption" sheetId="902" state="visible" r:id="rId902"/>
-    <sheet name="SyntheticData" sheetId="903" state="visible" r:id="rId903"/>
-    <sheet name="SystematicMonitoring" sheetId="904" state="visible" r:id="rId904"/>
-    <sheet name="TargetedAdvertising" sheetId="905" state="visible" r:id="rId905"/>
-    <sheet name="TechnicalMeasure" sheetId="906" state="visible" r:id="rId906"/>
-    <sheet name="TechnicalOrganisationalMeasure" sheetId="907" state="visible" r:id="rId907"/>
-    <sheet name="TechnicalServiceProvision" sheetId="908" state="visible" r:id="rId908"/>
-    <sheet name="TechnicalStandard" sheetId="909" state="visible" r:id="rId909"/>
-    <sheet name="Technology" sheetId="910" state="visible" r:id="rId910"/>
-    <sheet name="TemporalDuration" sheetId="911" state="visible" r:id="rId911"/>
-    <sheet name="TerminateContract" sheetId="912" state="visible" r:id="rId912"/>
-    <sheet name="TermsOfService" sheetId="913" state="visible" r:id="rId913"/>
-    <sheet name="ThirdCountry" sheetId="914" state="visible" r:id="rId914"/>
-    <sheet name="ThirdParty" sheetId="915" state="visible" r:id="rId915"/>
-    <sheet name="ThirdPartyAgreement" sheetId="916" state="visible" r:id="rId916"/>
-    <sheet name="ThirdPartyContract" sheetId="917" state="visible" r:id="rId917"/>
-    <sheet name="ThirdPartyDataSource" sheetId="918" state="visible" r:id="rId918"/>
-    <sheet name="ThirdPartySecurityProcedures" sheetId="919" state="visible" r:id="rId919"/>
-    <sheet name="Tourist" sheetId="920" state="visible" r:id="rId920"/>
-    <sheet name="Tracking" sheetId="921" state="visible" r:id="rId921"/>
-    <sheet name="TrackingByFirstParty" sheetId="922" state="visible" r:id="rId922"/>
-    <sheet name="TrackingByThirdParty" sheetId="923" state="visible" r:id="rId923"/>
-    <sheet name="Transfer" sheetId="924" state="visible" r:id="rId924"/>
-    <sheet name="Transform" sheetId="925" state="visible" r:id="rId925"/>
-    <sheet name="Transmit" sheetId="926" state="visible" r:id="rId926"/>
-    <sheet name="TrustedComputing" sheetId="927" state="visible" r:id="rId927"/>
-    <sheet name="TrustedExecutionEnvironment" sheetId="928" state="visible" r:id="rId928"/>
-    <sheet name="UnacceptableRule" sheetId="929" state="visible" r:id="rId929"/>
-    <sheet name="UncategorisedData" sheetId="930" state="visible" r:id="rId930"/>
-    <sheet name="Unexpected" sheetId="931" state="visible" r:id="rId931"/>
-    <sheet name="UninformedConsent" sheetId="932" state="visible" r:id="rId932"/>
-    <sheet name="Unintended" sheetId="933" state="visible" r:id="rId933"/>
-    <sheet name="UnknownApplicability" sheetId="934" state="visible" r:id="rId934"/>
-    <sheet name="Unlawful" sheetId="935" state="visible" r:id="rId935"/>
-    <sheet name="UnstructuredData" sheetId="936" state="visible" r:id="rId936"/>
-    <sheet name="UntilEventDuration" sheetId="937" state="visible" r:id="rId937"/>
-    <sheet name="UntilTimeDuration" sheetId="938" state="visible" r:id="rId938"/>
-    <sheet name="UnverifiedData" sheetId="939" state="visible" r:id="rId939"/>
-    <sheet name="UsageControl" sheetId="940" state="visible" r:id="rId940"/>
-    <sheet name="Use" sheetId="941" state="visible" r:id="rId941"/>
-    <sheet name="UseSyntheticData" sheetId="942" state="visible" r:id="rId942"/>
-    <sheet name="UserInterfacePersonalisation" sheetId="943" state="visible" r:id="rId943"/>
-    <sheet name="VariableLocation" sheetId="944" state="visible" r:id="rId944"/>
-    <sheet name="VendorManagement" sheetId="945" state="visible" r:id="rId945"/>
-    <sheet name="VendorPayment" sheetId="946" state="visible" r:id="rId946"/>
-    <sheet name="VendorRecordsManagement" sheetId="947" state="visible" r:id="rId947"/>
-    <sheet name="VendorSelectionAssessment" sheetId="948" state="visible" r:id="rId948"/>
-    <sheet name="Verification" sheetId="949" state="visible" r:id="rId949"/>
-    <sheet name="VerifiedData" sheetId="950" state="visible" r:id="rId950"/>
-    <sheet name="VirtualisationSecurity" sheetId="951" state="visible" r:id="rId951"/>
-    <sheet name="Visitor" sheetId="952" state="visible" r:id="rId952"/>
-    <sheet name="VitalInterest" sheetId="953" state="visible" r:id="rId953"/>
-    <sheet name="VitalInterestCompleted" sheetId="954" state="visible" r:id="rId954"/>
-    <sheet name="VitalInterestObjected" sheetId="955" state="visible" r:id="rId955"/>
-    <sheet name="VitalInterestOfDataSubject" sheetId="956" state="visible" r:id="rId956"/>
-    <sheet name="VitalInterestOfNaturalPerson" sheetId="957" state="visible" r:id="rId957"/>
-    <sheet name="VitalInterestOngoing" sheetId="958" state="visible" r:id="rId958"/>
-    <sheet name="VitalInterestPending" sheetId="959" state="visible" r:id="rId959"/>
-    <sheet name="VitalInterestStatus" sheetId="960" state="visible" r:id="rId960"/>
-    <sheet name="VulnerabilityTestingMethods" sheetId="961" state="visible" r:id="rId961"/>
-    <sheet name="VulnerableDataSubject" sheetId="962" state="visible" r:id="rId962"/>
-    <sheet name="VulnerableHuman" sheetId="963" state="visible" r:id="rId963"/>
-    <sheet name="WebBrowserSecurity" sheetId="964" state="visible" r:id="rId964"/>
-    <sheet name="WebSecurityProtocols" sheetId="965" state="visible" r:id="rId965"/>
-    <sheet name="WirelessSecurityProtocols" sheetId="966" state="visible" r:id="rId966"/>
-    <sheet name="WithdrawConsent" sheetId="967" state="visible" r:id="rId967"/>
-    <sheet name="WithdrawingFromProcess" sheetId="968" state="visible" r:id="rId968"/>
-    <sheet name="WithinDevice" sheetId="969" state="visible" r:id="rId969"/>
-    <sheet name="WithinPhysicalEnvironment" sheetId="970" state="visible" r:id="rId970"/>
-    <sheet name="WithinVirtualEnvironment" sheetId="971" state="visible" r:id="rId971"/>
-    <sheet name="ZeroKnowledgeAuthentication" sheetId="972" state="visible" r:id="rId972"/>
+    <sheet name="AcceptableRule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ActivelyInvolved" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ActivityCompleted" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ActivityHalted" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ActivityNotCompleted" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ActivityOngoing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ActivityPlanned" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ActivityProposed" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ActivityStatus" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Applicability" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AuditApproved" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="AuditConditionallyApproved" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="AuditNotRequired" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="AuditRejected" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="AuditRequested" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="AuditRequired" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="AuditStatus" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="AuthorityInformed" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="AuthorityUninformed" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="CompatibilityUnknown" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="ComplianceIndeterminate" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="ComplianceStatus" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="ComplianceUnknown" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="ComplianceViolation" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Compliant" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="ConformanceStatus" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Conformant" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Context" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="ContinuousFrequency" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="ControllerInformed" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="ControllerUninformed" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="DataSubjectInformed" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="DataSubjectUninformed" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="Deterrence" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="DeterrenceFollowed" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="DeterrenceNotFollowed" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="DpvDuration" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="DpvOptional" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="EndlessDuration" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="EntityInformed" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="EntityInformedStatus" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="EntityUninformed" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="ExpectationStatus" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Expected" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="FeeNotRequired" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="FeeRequired" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="FeeRequirement" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="FixedOccurrencesDuration" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="Frequency" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="Importance" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="IndeterminateDuration" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="Intended" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="IntentionStatus" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="InvolvementStatus" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="Justification" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="Lawful" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="Lawfulness" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="LawfulnessUnknown" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="LegalMeasure" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="Necessity" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="NonCompliant" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="NonConformant" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="NotApplicable" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="NotAvailable" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="NotInvolved" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="NotRequired" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="NotificationCompleted" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="NotificationFailed" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="NotificationNotNeeded" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="NotificationOngoing" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="NotificationPlanned" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="NotificationStatus" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="Obligation" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="ObligationFulfilled" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="ObligationUnfulfilled" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="ObligationViolated" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="OftenFrequency" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="OrganisationalMeasure" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="PartiallyCompliant" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="PassivelyInvolved" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="Permission" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="PermissionNotUtilised" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="PermissionUtilised" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="PhysicalMeasure" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="PrimaryImportance" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet name="PrimaryUse" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet name="Prohibition" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet name="ProhibitionUnviolated" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet name="ProhibitionViolated" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet name="RecipientInformed" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet name="RecipientUninformed" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet name="Recommendation" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet name="RecommendationFollowed" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet name="RecommendationNotFollowed" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet name="RequestAccepted" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet name="RequestAcknowledged" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="RequestActionDelayed" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet name="RequestFulfilled" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet name="RequestInitiated" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet name="RequestRejected" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet name="RequestRequiredActionPerformed" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet name="RequestRequiresAction" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet name="RequestStatus" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet name="RequestStatusQuery" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet name="RequestUnfulfilled" sheetId="105" state="visible" r:id="rId105"/>
+    <sheet name="Required" sheetId="106" state="visible" r:id="rId106"/>
+    <sheet name="ReuseCompatibility" sheetId="107" state="visible" r:id="rId107"/>
+    <sheet name="Rule" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet name="RuleFulfilled" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet name="RuleFulfilmentStatus" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet name="RuleUnfulfilled" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet name="RuleViolated" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet name="Scope" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet name="SecondaryImportance" sheetId="114" state="visible" r:id="rId114"/>
+    <sheet name="SecondaryUse" sheetId="115" state="visible" r:id="rId115"/>
+    <sheet name="SingularFrequency" sheetId="116" state="visible" r:id="rId116"/>
+    <sheet name="SporadicFrequency" sheetId="117" state="visible" r:id="rId117"/>
+    <sheet name="Status" sheetId="118" state="visible" r:id="rId118"/>
+    <sheet name="TechnicalMeasure" sheetId="119" state="visible" r:id="rId119"/>
+    <sheet name="TechnicalOrganisationalMeasure" sheetId="120" state="visible" r:id="rId120"/>
+    <sheet name="TemporalDuration" sheetId="121" state="visible" r:id="rId121"/>
+    <sheet name="UnacceptableRule" sheetId="122" state="visible" r:id="rId122"/>
+    <sheet name="Unexpected" sheetId="123" state="visible" r:id="rId123"/>
+    <sheet name="Unintended" sheetId="124" state="visible" r:id="rId124"/>
+    <sheet name="UnknownApplicability" sheetId="125" state="visible" r:id="rId125"/>
+    <sheet name="Unlawful" sheetId="126" state="visible" r:id="rId126"/>
+    <sheet name="UntilEventDuration" sheetId="127" state="visible" r:id="rId127"/>
+    <sheet name="UntilTimeDuration" sheetId="128" state="visible" r:id="rId128"/>
+    <sheet name="AcceptContract" sheetId="129" state="visible" r:id="rId129"/>
+    <sheet name="B2B2CContract" sheetId="130" state="visible" r:id="rId130"/>
+    <sheet name="B2BContract" sheetId="131" state="visible" r:id="rId131"/>
+    <sheet name="B2CContract" sheetId="132" state="visible" r:id="rId132"/>
+    <sheet name="C2BContract" sheetId="133" state="visible" r:id="rId133"/>
+    <sheet name="C2CContract" sheetId="134" state="visible" r:id="rId134"/>
+    <sheet name="City" sheetId="135" state="visible" r:id="rId135"/>
+    <sheet name="CloudLocation" sheetId="136" state="visible" r:id="rId136"/>
+    <sheet name="ConfidentialityAgreement" sheetId="137" state="visible" r:id="rId137"/>
+    <sheet name="Consent" sheetId="138" state="visible" r:id="rId138"/>
+    <sheet name="ConsumerStandardFormContract" sheetId="139" state="visible" r:id="rId139"/>
+    <sheet name="Contract" sheetId="140" state="visible" r:id="rId140"/>
+    <sheet name="ContractActivationStatus" sheetId="141" state="visible" r:id="rId141"/>
+    <sheet name="ContractActive" sheetId="142" state="visible" r:id="rId142"/>
+    <sheet name="ContractAmended" sheetId="143" state="visible" r:id="rId143"/>
+    <sheet name="ContractAmendmentClause" sheetId="144" state="visible" r:id="rId144"/>
+    <sheet name="ContractApproved" sheetId="145" state="visible" r:id="rId145"/>
+    <sheet name="ContractBeingPerformed" sheetId="146" state="visible" r:id="rId146"/>
+    <sheet name="ContractBreached" sheetId="147" state="visible" r:id="rId147"/>
+    <sheet name="ContractByDomain" sheetId="148" state="visible" r:id="rId148"/>
+    <sheet name="ContractByEntityType" sheetId="149" state="visible" r:id="rId149"/>
+    <sheet name="ContractByNegotiationType" sheetId="150" state="visible" r:id="rId150"/>
+    <sheet name="ContractConfidentialityClause" sheetId="151" state="visible" r:id="rId151"/>
+    <sheet name="ContractControl" sheetId="152" state="visible" r:id="rId152"/>
+    <sheet name="ContractDefinitions" sheetId="153" state="visible" r:id="rId153"/>
+    <sheet name="ContractDisputeResolutionClause" sheetId="154" state="visible" r:id="rId154"/>
+    <sheet name="ContractDisputed" sheetId="155" state="visible" r:id="rId155"/>
+    <sheet name="ContractDrafted" sheetId="156" state="visible" r:id="rId156"/>
+    <sheet name="ContractExecutionStatus" sheetId="157" state="visible" r:id="rId157"/>
+    <sheet name="ContractExpired" sheetId="158" state="visible" r:id="rId158"/>
+    <sheet name="ContractExtended" sheetId="159" state="visible" r:id="rId159"/>
+    <sheet name="ContractFulfilled" sheetId="160" state="visible" r:id="rId160"/>
+    <sheet name="ContractFulfilmentStatus" sheetId="161" state="visible" r:id="rId161"/>
+    <sheet name="ContractFullyExecuted" sheetId="162" state="visible" r:id="rId162"/>
+    <sheet name="ContractFullySigned" sheetId="163" state="visible" r:id="rId163"/>
+    <sheet name="ContractInactive" sheetId="164" state="visible" r:id="rId164"/>
+    <sheet name="ContractJurisdictionClause" sheetId="165" state="visible" r:id="rId165"/>
+    <sheet name="ContractNegotiated" sheetId="166" state="visible" r:id="rId166"/>
+    <sheet name="ContractNotFulfilled" sheetId="167" state="visible" r:id="rId167"/>
+    <sheet name="ContractOffered" sheetId="168" state="visible" r:id="rId168"/>
+    <sheet name="ContractPartiallyFulfilled" sheetId="169" state="visible" r:id="rId169"/>
+    <sheet name="ContractPartiallySigned" sheetId="170" state="visible" r:id="rId170"/>
+    <sheet name="ContractPerformance" sheetId="171" state="visible" r:id="rId171"/>
+    <sheet name="ContractPerformanceStatus" sheetId="172" state="visible" r:id="rId172"/>
+    <sheet name="ContractPreamble" sheetId="173" state="visible" r:id="rId173"/>
+    <sheet name="ContractPreparationStatus" sheetId="174" state="visible" r:id="rId174"/>
+    <sheet name="ContractRejected" sheetId="175" state="visible" r:id="rId175"/>
+    <sheet name="ContractRenewed" sheetId="176" state="visible" r:id="rId176"/>
+    <sheet name="ContractSignedByParty" sheetId="177" state="visible" r:id="rId177"/>
+    <sheet name="ContractStatus" sheetId="178" state="visible" r:id="rId178"/>
+    <sheet name="ContractTemporarilySuspended" sheetId="179" state="visible" r:id="rId179"/>
+    <sheet name="ContractTerminated" sheetId="180" state="visible" r:id="rId180"/>
+    <sheet name="ContractTerminationClause" sheetId="181" state="visible" r:id="rId181"/>
+    <sheet name="ContractTerminationStatus" sheetId="182" state="visible" r:id="rId182"/>
+    <sheet name="ContractUnderNegotiation" sheetId="183" state="visible" r:id="rId183"/>
+    <sheet name="ContractUnderReview" sheetId="184" state="visible" r:id="rId184"/>
+    <sheet name="ContractViolated" sheetId="185" state="visible" r:id="rId185"/>
+    <sheet name="ContractualClause" sheetId="186" state="visible" r:id="rId186"/>
+    <sheet name="ContractualClauseFulfilled" sheetId="187" state="visible" r:id="rId187"/>
+    <sheet name="ContractualClauseFulfilmentStatus" sheetId="188" state="visible" r:id="rId188"/>
+    <sheet name="ContractualClauseNotFulfilled" sheetId="189" state="visible" r:id="rId189"/>
+    <sheet name="ContractualClausePartiallyFulfilled" sheetId="190" state="visible" r:id="rId190"/>
+    <sheet name="ContractualClauseViolated" sheetId="191" state="visible" r:id="rId191"/>
+    <sheet name="ContractualTerms" sheetId="192" state="visible" r:id="rId192"/>
+    <sheet name="ControllerDataSubjectAgreement" sheetId="193" state="visible" r:id="rId193"/>
+    <sheet name="ControllerProcessorAgreement" sheetId="194" state="visible" r:id="rId194"/>
+    <sheet name="DataControllerContract" sheetId="195" state="visible" r:id="rId195"/>
+    <sheet name="DataHandlingClause" sheetId="196" state="visible" r:id="rId196"/>
+    <sheet name="DataProcessingAgreement" sheetId="197" state="visible" r:id="rId197"/>
+    <sheet name="DataProcessorContract" sheetId="198" state="visible" r:id="rId198"/>
+    <sheet name="DataSubjectContract" sheetId="199" state="visible" r:id="rId199"/>
+    <sheet name="DataTransferLegalBasis" sheetId="200" state="visible" r:id="rId200"/>
+    <sheet name="DecentralisedLocations" sheetId="201" state="visible" r:id="rId201"/>
+    <sheet name="DistributionAgreement" sheetId="202" state="visible" r:id="rId202"/>
+    <sheet name="DpvCountry" sheetId="203" state="visible" r:id="rId203"/>
+    <sheet name="DpvJurisdiction" sheetId="204" state="visible" r:id="rId204"/>
+    <sheet name="DpvLocation" sheetId="205" state="visible" r:id="rId205"/>
+    <sheet name="DpvRegion" sheetId="206" state="visible" r:id="rId206"/>
+    <sheet name="EULA" sheetId="207" state="visible" r:id="rId207"/>
+    <sheet name="EconomicUnion" sheetId="208" state="visible" r:id="rId208"/>
+    <sheet name="EmploymentContract" sheetId="209" state="visible" r:id="rId209"/>
+    <sheet name="EnterIntoContract" sheetId="210" state="visible" r:id="rId210"/>
+    <sheet name="FederatedLocations" sheetId="211" state="visible" r:id="rId211"/>
+    <sheet name="FixedLocation" sheetId="212" state="visible" r:id="rId212"/>
+    <sheet name="FixedMultipleLocations" sheetId="213" state="visible" r:id="rId213"/>
+    <sheet name="FixedSingularLocation" sheetId="214" state="visible" r:id="rId214"/>
+    <sheet name="G2BContract" sheetId="215" state="visible" r:id="rId215"/>
+    <sheet name="G2CContract" sheetId="216" state="visible" r:id="rId216"/>
+    <sheet name="G2GContract" sheetId="217" state="visible" r:id="rId217"/>
+    <sheet name="HybridPublicPrivateSpace" sheetId="218" state="visible" r:id="rId218"/>
+    <sheet name="InverseJurisdiction" sheetId="219" state="visible" r:id="rId219"/>
+    <sheet name="JointDataControllersAgreement" sheetId="220" state="visible" r:id="rId220"/>
+    <sheet name="Law" sheetId="221" state="visible" r:id="rId221"/>
+    <sheet name="LegalAgreement" sheetId="222" state="visible" r:id="rId222"/>
+    <sheet name="LegalBasis" sheetId="223" state="visible" r:id="rId223"/>
+    <sheet name="LegalObligation" sheetId="224" state="visible" r:id="rId224"/>
+    <sheet name="LegalObligationCompleted" sheetId="225" state="visible" r:id="rId225"/>
+    <sheet name="LegalObligationOngoing" sheetId="226" state="visible" r:id="rId226"/>
+    <sheet name="LegalObligationPending" sheetId="227" state="visible" r:id="rId227"/>
+    <sheet name="LegalObligationStatus" sheetId="228" state="visible" r:id="rId228"/>
+    <sheet name="LegitimateInterest" sheetId="229" state="visible" r:id="rId229"/>
+    <sheet name="LegitimateInterestInformed" sheetId="230" state="visible" r:id="rId230"/>
+    <sheet name="LegitimateInterestNotObjected" sheetId="231" state="visible" r:id="rId231"/>
+    <sheet name="LegitimateInterestObjected" sheetId="232" state="visible" r:id="rId232"/>
+    <sheet name="LegitimateInterestOfController" sheetId="233" state="visible" r:id="rId233"/>
+    <sheet name="LegitimateInterestOfDataSubject" sheetId="234" state="visible" r:id="rId234"/>
+    <sheet name="LegitimateInterestOfThirdParty" sheetId="235" state="visible" r:id="rId235"/>
+    <sheet name="LegitimateInterestStatus" sheetId="236" state="visible" r:id="rId236"/>
+    <sheet name="LegitimateInterestUninformed" sheetId="237" state="visible" r:id="rId237"/>
+    <sheet name="LicenseAgreement" sheetId="238" state="visible" r:id="rId238"/>
+    <sheet name="LocalLocation" sheetId="239" state="visible" r:id="rId239"/>
+    <sheet name="LocationFixture" sheetId="240" state="visible" r:id="rId240"/>
+    <sheet name="LocationLocality" sheetId="241" state="visible" r:id="rId241"/>
+    <sheet name="NDA" sheetId="242" state="visible" r:id="rId242"/>
+    <sheet name="NegotiateContract" sheetId="243" state="visible" r:id="rId243"/>
+    <sheet name="NegotiatedContract" sheetId="244" state="visible" r:id="rId244"/>
+    <sheet name="OfferContract" sheetId="245" state="visible" r:id="rId245"/>
+    <sheet name="OfficialAuthorityExerciseCompleted" sheetId="246" state="visible" r:id="rId246"/>
+    <sheet name="OfficialAuthorityExerciseOngoing" sheetId="247" state="visible" r:id="rId247"/>
+    <sheet name="OfficialAuthorityExercisePending" sheetId="248" state="visible" r:id="rId248"/>
+    <sheet name="OfficialAuthorityExerciseStatus" sheetId="249" state="visible" r:id="rId249"/>
+    <sheet name="OfficialAuthorityOfController" sheetId="250" state="visible" r:id="rId250"/>
+    <sheet name="PersonalSpace" sheetId="251" state="visible" r:id="rId251"/>
+    <sheet name="PrivateCommunalSpace" sheetId="252" state="visible" r:id="rId252"/>
+    <sheet name="PrivateLocation" sheetId="253" state="visible" r:id="rId253"/>
+    <sheet name="PrivateSpace" sheetId="254" state="visible" r:id="rId254"/>
+    <sheet name="PrivatelyOperatedPublicSpace" sheetId="255" state="visible" r:id="rId255"/>
+    <sheet name="PrivatelyOwnedPublicSpace" sheetId="256" state="visible" r:id="rId256"/>
+    <sheet name="PrivatelyOwnedSpace" sheetId="257" state="visible" r:id="rId257"/>
+    <sheet name="ProviderStandardFormContract" sheetId="258" state="visible" r:id="rId258"/>
+    <sheet name="PublicInterest" sheetId="259" state="visible" r:id="rId259"/>
+    <sheet name="PublicInterestCompleted" sheetId="260" state="visible" r:id="rId260"/>
+    <sheet name="PublicInterestObjected" sheetId="261" state="visible" r:id="rId261"/>
+    <sheet name="PublicInterestOngoing" sheetId="262" state="visible" r:id="rId262"/>
+    <sheet name="PublicInterestPending" sheetId="263" state="visible" r:id="rId263"/>
+    <sheet name="PublicInterestStatus" sheetId="264" state="visible" r:id="rId264"/>
+    <sheet name="PublicLocation" sheetId="265" state="visible" r:id="rId265"/>
+    <sheet name="PublicSpace" sheetId="266" state="visible" r:id="rId266"/>
+    <sheet name="PubliclyAccessibleSpace" sheetId="267" state="visible" r:id="rId267"/>
+    <sheet name="PubliclyOwnedSpace" sheetId="268" state="visible" r:id="rId268"/>
+    <sheet name="RandomLocation" sheetId="269" state="visible" r:id="rId269"/>
+    <sheet name="RefuseContract" sheetId="270" state="visible" r:id="rId270"/>
+    <sheet name="RemoteLocation" sheetId="271" state="visible" r:id="rId271"/>
+    <sheet name="SemiPrivateSpace" sheetId="272" state="visible" r:id="rId272"/>
+    <sheet name="ServiceLevelAgreement" sheetId="273" state="visible" r:id="rId273"/>
+    <sheet name="StandardFormContract" sheetId="274" state="visible" r:id="rId274"/>
+    <sheet name="StatisticalConfidentialityAgreement" sheetId="275" state="visible" r:id="rId275"/>
+    <sheet name="SubProcessorAgreement" sheetId="276" state="visible" r:id="rId276"/>
+    <sheet name="SupraNationalUnion" sheetId="277" state="visible" r:id="rId277"/>
+    <sheet name="TerminateContract" sheetId="278" state="visible" r:id="rId278"/>
+    <sheet name="TermsOfService" sheetId="279" state="visible" r:id="rId279"/>
+    <sheet name="ThirdCountry" sheetId="280" state="visible" r:id="rId280"/>
+    <sheet name="ThirdPartyAgreement" sheetId="281" state="visible" r:id="rId281"/>
+    <sheet name="ThirdPartyContract" sheetId="282" state="visible" r:id="rId282"/>
+    <sheet name="VariableLocation" sheetId="283" state="visible" r:id="rId283"/>
+    <sheet name="VitalInterest" sheetId="284" state="visible" r:id="rId284"/>
+    <sheet name="VitalInterestCompleted" sheetId="285" state="visible" r:id="rId285"/>
+    <sheet name="VitalInterestObjected" sheetId="286" state="visible" r:id="rId286"/>
+    <sheet name="VitalInterestOfDataSubject" sheetId="287" state="visible" r:id="rId287"/>
+    <sheet name="VitalInterestOfNaturalPerson" sheetId="288" state="visible" r:id="rId288"/>
+    <sheet name="VitalInterestOngoing" sheetId="289" state="visible" r:id="rId289"/>
+    <sheet name="VitalInterestPending" sheetId="290" state="visible" r:id="rId290"/>
+    <sheet name="VitalInterestStatus" sheetId="291" state="visible" r:id="rId291"/>
+    <sheet name="WithinDevice" sheetId="292" state="visible" r:id="rId292"/>
+    <sheet name="WithinPhysicalEnvironment" sheetId="293" state="visible" r:id="rId293"/>
+    <sheet name="WithinVirtualEnvironment" sheetId="294" state="visible" r:id="rId294"/>
+    <sheet name="AcademicScientificOrganisation" sheetId="295" state="visible" r:id="rId295"/>
+    <sheet name="Adult" sheetId="296" state="visible" r:id="rId296"/>
+    <sheet name="AmbulanceProvider" sheetId="297" state="visible" r:id="rId297"/>
+    <sheet name="Applicant" sheetId="298" state="visible" r:id="rId298"/>
+    <sheet name="AsylumSeeker" sheetId="299" state="visible" r:id="rId299"/>
+    <sheet name="CharityOrganisation" sheetId="300" state="visible" r:id="rId300"/>
+    <sheet name="Child" sheetId="301" state="visible" r:id="rId301"/>
+    <sheet name="Citizen" sheetId="302" state="visible" r:id="rId302"/>
+    <sheet name="Client" sheetId="303" state="visible" r:id="rId303"/>
+    <sheet name="Clinic" sheetId="304" state="visible" r:id="rId304"/>
+    <sheet name="DataController" sheetId="305" state="visible" r:id="rId305"/>
+    <sheet name="DataExporter" sheetId="306" state="visible" r:id="rId306"/>
+    <sheet name="DataImporter" sheetId="307" state="visible" r:id="rId307"/>
+    <sheet name="DataProcessor" sheetId="308" state="visible" r:id="rId308"/>
+    <sheet name="DataProtectionAuthority" sheetId="309" state="visible" r:id="rId309"/>
+    <sheet name="DataProtectionOfficer" sheetId="310" state="visible" r:id="rId310"/>
+    <sheet name="DataSubProcessor" sheetId="311" state="visible" r:id="rId311"/>
+    <sheet name="DataSubject" sheetId="312" state="visible" r:id="rId312"/>
+    <sheet name="DpvAgent" sheetId="313" state="visible" r:id="rId313"/>
+    <sheet name="DpvAuthority" sheetId="314" state="visible" r:id="rId314"/>
+    <sheet name="DpvConsumer" sheetId="315" state="visible" r:id="rId315"/>
+    <sheet name="DpvCustomer" sheetId="316" state="visible" r:id="rId316"/>
+    <sheet name="DpvEntity" sheetId="317" state="visible" r:id="rId317"/>
+    <sheet name="DpvOrganisation" sheetId="318" state="visible" r:id="rId318"/>
+    <sheet name="DpvRecipient" sheetId="319" state="visible" r:id="rId319"/>
+    <sheet name="DpvUser" sheetId="320" state="visible" r:id="rId320"/>
+    <sheet name="EducationalOrganisation" sheetId="321" state="visible" r:id="rId321"/>
+    <sheet name="ElderlyDataSubject" sheetId="322" state="visible" r:id="rId322"/>
+    <sheet name="ElderlyHuman" sheetId="323" state="visible" r:id="rId323"/>
+    <sheet name="EmergencyHealthcareProvider" sheetId="324" state="visible" r:id="rId324"/>
+    <sheet name="EmergencyServiceProvider" sheetId="325" state="visible" r:id="rId325"/>
+    <sheet name="Employee" sheetId="326" state="visible" r:id="rId326"/>
+    <sheet name="FireDepartment" sheetId="327" state="visible" r:id="rId327"/>
+    <sheet name="ForProfitOrganisation" sheetId="328" state="visible" r:id="rId328"/>
+    <sheet name="GovernmentalOrganisation" sheetId="329" state="visible" r:id="rId329"/>
+    <sheet name="GuardianOfDataSubject" sheetId="330" state="visible" r:id="rId330"/>
+    <sheet name="GuardianOfHuman" sheetId="331" state="visible" r:id="rId331"/>
+    <sheet name="HealthcareOrganisation" sheetId="332" state="visible" r:id="rId332"/>
+    <sheet name="Hospital" sheetId="333" state="visible" r:id="rId333"/>
+    <sheet name="HumanSubject" sheetId="334" state="visible" r:id="rId334"/>
+    <sheet name="Immigrant" sheetId="335" state="visible" r:id="rId335"/>
+    <sheet name="IndustryConsortium" sheetId="336" state="visible" r:id="rId336"/>
+    <sheet name="InternationalOrganisation" sheetId="337" state="visible" r:id="rId337"/>
+    <sheet name="JobApplicant" sheetId="338" state="visible" r:id="rId338"/>
+    <sheet name="JointDataControllers" sheetId="339" state="visible" r:id="rId339"/>
+    <sheet name="JudicialOrganisation" sheetId="340" state="visible" r:id="rId340"/>
+    <sheet name="LawEnforcementOrganisation" sheetId="341" state="visible" r:id="rId341"/>
+    <sheet name="LegalAgent" sheetId="342" state="visible" r:id="rId342"/>
+    <sheet name="LegalEntity" sheetId="343" state="visible" r:id="rId343"/>
+    <sheet name="Member" sheetId="344" state="visible" r:id="rId344"/>
+    <sheet name="MentallyVulnerableDataSubject" sheetId="345" state="visible" r:id="rId345"/>
+    <sheet name="MentallyVulnerableHuman" sheetId="346" state="visible" r:id="rId346"/>
+    <sheet name="NationalAuthority" sheetId="347" state="visible" r:id="rId347"/>
+    <sheet name="NaturalPerson" sheetId="348" state="visible" r:id="rId348"/>
+    <sheet name="NonCitizen" sheetId="349" state="visible" r:id="rId349"/>
+    <sheet name="NonGovernmentalOrganisation" sheetId="350" state="visible" r:id="rId350"/>
+    <sheet name="NonProfitOrganisation" sheetId="351" state="visible" r:id="rId351"/>
+    <sheet name="OrganisationalUnit" sheetId="352" state="visible" r:id="rId352"/>
+    <sheet name="ParentLegalEntity" sheetId="353" state="visible" r:id="rId353"/>
+    <sheet name="ParentOfDataSubject" sheetId="354" state="visible" r:id="rId354"/>
+    <sheet name="ParentOfHuman" sheetId="355" state="visible" r:id="rId355"/>
+    <sheet name="Participant" sheetId="356" state="visible" r:id="rId356"/>
+    <sheet name="Patient" sheetId="357" state="visible" r:id="rId357"/>
+    <sheet name="PrivateSectorBody" sheetId="358" state="visible" r:id="rId358"/>
+    <sheet name="PublicRegisterOfEntities" sheetId="359" state="visible" r:id="rId359"/>
+    <sheet name="PublicSectorBody" sheetId="360" state="visible" r:id="rId360"/>
+    <sheet name="RegionalAuthority" sheetId="361" state="visible" r:id="rId361"/>
+    <sheet name="ReligiousAssociations" sheetId="362" state="visible" r:id="rId362"/>
+    <sheet name="Representative" sheetId="363" state="visible" r:id="rId363"/>
+    <sheet name="SMEOrganisation" sheetId="364" state="visible" r:id="rId364"/>
+    <sheet name="ServiceConsumer" sheetId="365" state="visible" r:id="rId365"/>
+    <sheet name="ServiceProvider" sheetId="366" state="visible" r:id="rId366"/>
+    <sheet name="StartupOrganisation" sheetId="367" state="visible" r:id="rId367"/>
+    <sheet name="Student" sheetId="368" state="visible" r:id="rId368"/>
+    <sheet name="Subscriber" sheetId="369" state="visible" r:id="rId369"/>
+    <sheet name="SubsidiaryLegalEntity" sheetId="370" state="visible" r:id="rId370"/>
+    <sheet name="SupraNationalAuthority" sheetId="371" state="visible" r:id="rId371"/>
+    <sheet name="ThirdParty" sheetId="372" state="visible" r:id="rId372"/>
+    <sheet name="Tourist" sheetId="373" state="visible" r:id="rId373"/>
+    <sheet name="Visitor" sheetId="374" state="visible" r:id="rId374"/>
+    <sheet name="VulnerableDataSubject" sheetId="375" state="visible" r:id="rId375"/>
+    <sheet name="VulnerableHuman" sheetId="376" state="visible" r:id="rId376"/>
+    <sheet name="AIGovernance" sheetId="377" state="visible" r:id="rId377"/>
+    <sheet name="AILiteracy" sheetId="378" state="visible" r:id="rId378"/>
+    <sheet name="AINotice" sheetId="379" state="visible" r:id="rId379"/>
+    <sheet name="AcceptableUsePolicy" sheetId="380" state="visible" r:id="rId380"/>
+    <sheet name="AccessControlMethod" sheetId="381" state="visible" r:id="rId381"/>
+    <sheet name="ActivityMonitoring" sheetId="382" state="visible" r:id="rId382"/>
+    <sheet name="Anonymisation" sheetId="383" state="visible" r:id="rId383"/>
+    <sheet name="AnonymisedData" sheetId="384" state="visible" r:id="rId384"/>
+    <sheet name="ApprovalProcedure" sheetId="385" state="visible" r:id="rId385"/>
+    <sheet name="Assessment" sheetId="386" state="visible" r:id="rId386"/>
+    <sheet name="AssetManagementProcedures" sheetId="387" state="visible" r:id="rId387"/>
+    <sheet name="AsymmetricCryptography" sheetId="388" state="visible" r:id="rId388"/>
+    <sheet name="AsymmetricEncryption" sheetId="389" state="visible" r:id="rId389"/>
+    <sheet name="Audit" sheetId="390" state="visible" r:id="rId390"/>
+    <sheet name="AuthenticationABC" sheetId="391" state="visible" r:id="rId391"/>
+    <sheet name="AuthenticationPABC" sheetId="392" state="visible" r:id="rId392"/>
+    <sheet name="AuthenticationProtocols" sheetId="393" state="visible" r:id="rId393"/>
+    <sheet name="AuthorisationProcedure" sheetId="394" state="visible" r:id="rId394"/>
+    <sheet name="AuthorisationProtocols" sheetId="395" state="visible" r:id="rId395"/>
+    <sheet name="BackgroundChecks" sheetId="396" state="visible" r:id="rId396"/>
+    <sheet name="BiometricAuthentication" sheetId="397" state="visible" r:id="rId397"/>
+    <sheet name="Certification" sheetId="398" state="visible" r:id="rId398"/>
+    <sheet name="CertificationSeal" sheetId="399" state="visible" r:id="rId399"/>
+    <sheet name="CodeOfConduct" sheetId="400" state="visible" r:id="rId400"/>
+    <sheet name="CollectedData" sheetId="401" state="visible" r:id="rId401"/>
+    <sheet name="CollectedPersonalData" sheetId="402" state="visible" r:id="rId402"/>
+    <sheet name="CommerciallyConfidentialData" sheetId="403" state="visible" r:id="rId403"/>
+    <sheet name="ComplianceAssessment" sheetId="404" state="visible" r:id="rId404"/>
+    <sheet name="ComplianceMonitoring" sheetId="405" state="visible" r:id="rId405"/>
+    <sheet name="ConfidentialData" sheetId="406" state="visible" r:id="rId406"/>
+    <sheet name="ConformanceAssessment" sheetId="407" state="visible" r:id="rId407"/>
+    <sheet name="ConsentManagement" sheetId="408" state="visible" r:id="rId408"/>
+    <sheet name="ConsentReceipt" sheetId="409" state="visible" r:id="rId409"/>
+    <sheet name="ConsentRecord" sheetId="410" state="visible" r:id="rId410"/>
+    <sheet name="Consultation" sheetId="411" state="visible" r:id="rId411"/>
+    <sheet name="ConsultationWithAuthority" sheetId="412" state="visible" r:id="rId412"/>
+    <sheet name="ConsultationWithDPO" sheetId="413" state="visible" r:id="rId413"/>
+    <sheet name="ConsultationWithDataSubject" sheetId="414" state="visible" r:id="rId414"/>
+    <sheet name="ConsultationWithDataSubjectRepresentative" sheetId="415" state="visible" r:id="rId415"/>
+    <sheet name="ContextuallyAnonymisedData" sheetId="416" state="visible" r:id="rId416"/>
+    <sheet name="CredentialManagement" sheetId="417" state="visible" r:id="rId417"/>
+    <sheet name="CryptographicAuthentication" sheetId="418" state="visible" r:id="rId418"/>
+    <sheet name="CryptographicKeyManagement" sheetId="419" state="visible" r:id="rId419"/>
+    <sheet name="CryptographicMethods" sheetId="420" state="visible" r:id="rId420"/>
+    <sheet name="CybersecurityTraining" sheetId="421" state="visible" r:id="rId421"/>
+    <sheet name="DataAvailabilityAssessment" sheetId="422" state="visible" r:id="rId422"/>
+    <sheet name="DataBackupProtocols" sheetId="423" state="visible" r:id="rId423"/>
+    <sheet name="DataBreachNotification" sheetId="424" state="visible" r:id="rId424"/>
+    <sheet name="DataBreachRecord" sheetId="425" state="visible" r:id="rId425"/>
+    <sheet name="DataDeletionPolicy" sheetId="426" state="visible" r:id="rId426"/>
+    <sheet name="DataErasurePolicy" sheetId="427" state="visible" r:id="rId427"/>
+    <sheet name="DataGovernance" sheetId="428" state="visible" r:id="rId428"/>
+    <sheet name="DataInteroperabilityAssessment" sheetId="429" state="visible" r:id="rId429"/>
+    <sheet name="DataInteroperabilityImprovement" sheetId="430" state="visible" r:id="rId430"/>
+    <sheet name="DataInteroperabilityManagement" sheetId="431" state="visible" r:id="rId431"/>
+    <sheet name="DataInventoryManagement" sheetId="432" state="visible" r:id="rId432"/>
+    <sheet name="DataJurisdictionPolicy" sheetId="433" state="visible" r:id="rId433"/>
+    <sheet name="DataLiteracy" sheetId="434" state="visible" r:id="rId434"/>
+    <sheet name="DataProcessingPolicy" sheetId="435" state="visible" r:id="rId435"/>
+    <sheet name="DataProcessingRecord" sheetId="436" state="visible" r:id="rId436"/>
+    <sheet name="DataProtectionTraining" sheetId="437" state="visible" r:id="rId437"/>
+    <sheet name="DataQualityAssessment" sheetId="438" state="visible" r:id="rId438"/>
+    <sheet name="DataQualityImprovement" sheetId="439" state="visible" r:id="rId439"/>
+    <sheet name="DataQualityManagement" sheetId="440" state="visible" r:id="rId440"/>
+    <sheet name="DataRedaction" sheetId="441" state="visible" r:id="rId441"/>
+    <sheet name="DataRestorationPolicy" sheetId="442" state="visible" r:id="rId442"/>
+    <sheet name="DataReusePolicy" sheetId="443" state="visible" r:id="rId443"/>
+    <sheet name="DataSanitisationTechnique" sheetId="444" state="visible" r:id="rId444"/>
+    <sheet name="DataSecurityManagement" sheetId="445" state="visible" r:id="rId445"/>
+    <sheet name="DataStoragePolicy" sheetId="446" state="visible" r:id="rId446"/>
+    <sheet name="DataSubjectRightsManagement" sheetId="447" state="visible" r:id="rId447"/>
+    <sheet name="DataSuitabilityAssessment" sheetId="448" state="visible" r:id="rId448"/>
+    <sheet name="DataTransferRecord" sheetId="449" state="visible" r:id="rId449"/>
+    <sheet name="Deidentification" sheetId="450" state="visible" r:id="rId450"/>
+    <sheet name="DerivedData" sheetId="451" state="visible" r:id="rId451"/>
+    <sheet name="DerivedPersonalData" sheetId="452" state="visible" r:id="rId452"/>
+    <sheet name="DesignStandard" sheetId="453" state="visible" r:id="rId453"/>
+    <sheet name="DeterministicPseudonymisation" sheetId="454" state="visible" r:id="rId454"/>
+    <sheet name="DifferentialPrivacy" sheetId="455" state="visible" r:id="rId455"/>
+    <sheet name="DigitalLiteracy" sheetId="456" state="visible" r:id="rId456"/>
+    <sheet name="DigitalRightsManagement" sheetId="457" state="visible" r:id="rId457"/>
+    <sheet name="DigitalSignatures" sheetId="458" state="visible" r:id="rId458"/>
+    <sheet name="DisasterRecoveryProcedures" sheetId="459" state="visible" r:id="rId459"/>
+    <sheet name="DistributedSystemSecurity" sheetId="460" state="visible" r:id="rId460"/>
+    <sheet name="DocumentRandomisedPseudonymisation" sheetId="461" state="visible" r:id="rId461"/>
+    <sheet name="DocumentSecurity" sheetId="462" state="visible" r:id="rId462"/>
+    <sheet name="DpvData" sheetId="463" state="visible" r:id="rId463"/>
+    <sheet name="EducationalTraining" sheetId="464" state="visible" r:id="rId464"/>
+    <sheet name="EffectivenessDeterminationProcedures" sheetId="465" state="visible" r:id="rId465"/>
+    <sheet name="Encryption" sheetId="466" state="visible" r:id="rId466"/>
+    <sheet name="EncryptionAtRest" sheetId="467" state="visible" r:id="rId467"/>
+    <sheet name="EncryptionInTransfer" sheetId="468" state="visible" r:id="rId468"/>
+    <sheet name="EncryptionInUse" sheetId="469" state="visible" r:id="rId469"/>
+    <sheet name="EndToEndEncryption" sheetId="470" state="visible" r:id="rId470"/>
+    <sheet name="EnvironmentalProtection" sheetId="471" state="visible" r:id="rId471"/>
+    <sheet name="FailSafeProtocols" sheetId="472" state="visible" r:id="rId472"/>
+    <sheet name="FileSystemSecurity" sheetId="473" state="visible" r:id="rId473"/>
+    <sheet name="FullyRandomisedPseudonymisation" sheetId="474" state="visible" r:id="rId474"/>
+    <sheet name="GeneratedData" sheetId="475" state="visible" r:id="rId475"/>
+    <sheet name="GeneratedPersonalData" sheetId="476" state="visible" r:id="rId476"/>
+    <sheet name="GovernanceProcedures" sheetId="477" state="visible" r:id="rId477"/>
+    <sheet name="Guideline" sheetId="478" state="visible" r:id="rId478"/>
+    <sheet name="GuidelinesPrinciple" sheetId="479" state="visible" r:id="rId479"/>
+    <sheet name="HardwareSecurityProtocols" sheetId="480" state="visible" r:id="rId480"/>
+    <sheet name="HashFunctions" sheetId="481" state="visible" r:id="rId481"/>
+    <sheet name="HashMessageAuthenticationCode" sheetId="482" state="visible" r:id="rId482"/>
+    <sheet name="HomomorphicEncryption" sheetId="483" state="visible" r:id="rId483"/>
+    <sheet name="HumanOversight" sheetId="484" state="visible" r:id="rId484"/>
+    <sheet name="IPRManagement" sheetId="485" state="visible" r:id="rId485"/>
+    <sheet name="IdentifyingPersonalData" sheetId="486" state="visible" r:id="rId486"/>
+    <sheet name="IdentityManagementMethod" sheetId="487" state="visible" r:id="rId487"/>
+    <sheet name="IncidentManagementProcedures" sheetId="488" state="visible" r:id="rId488"/>
+    <sheet name="IncidentReportingCommunication" sheetId="489" state="visible" r:id="rId489"/>
+    <sheet name="IncorrectData" sheetId="490" state="visible" r:id="rId490"/>
+    <sheet name="InferredData" sheetId="491" state="visible" r:id="rId491"/>
+    <sheet name="InferredPersonalData" sheetId="492" state="visible" r:id="rId492"/>
+    <sheet name="InformationAudit" sheetId="493" state="visible" r:id="rId493"/>
+    <sheet name="InformationFlowControl" sheetId="494" state="visible" r:id="rId494"/>
+    <sheet name="InformationSecurityPolicy" sheetId="495" state="visible" r:id="rId495"/>
+    <sheet name="IntellectualPropertyData" sheetId="496" state="visible" r:id="rId496"/>
+    <sheet name="IntrusionDetectionSystem" sheetId="497" state="visible" r:id="rId497"/>
+    <sheet name="LegalComplianceAssessment" sheetId="498" state="visible" r:id="rId498"/>
+    <sheet name="LegalComplianceAudit" sheetId="499" state="visible" r:id="rId499"/>
+    <sheet name="LegitimateInterestAssessment" sheetId="500" state="visible" r:id="rId500"/>
+    <sheet name="LoggingPolicy" sheetId="501" state="visible" r:id="rId501"/>
+    <sheet name="ManagementStandard" sheetId="502" state="visible" r:id="rId502"/>
+    <sheet name="MessageAuthenticationCodes" sheetId="503" state="visible" r:id="rId503"/>
+    <sheet name="MetadataManagement" sheetId="504" state="visible" r:id="rId504"/>
+    <sheet name="MobilePlatformSecurity" sheetId="505" state="visible" r:id="rId505"/>
+    <sheet name="MonitoringPolicy" sheetId="506" state="visible" r:id="rId506"/>
+    <sheet name="MonotonicCounterPseudonymisation" sheetId="507" state="visible" r:id="rId507"/>
+    <sheet name="MultiFactorAuthentication" sheetId="508" state="visible" r:id="rId508"/>
+    <sheet name="NetworkProxyRouting" sheetId="509" state="visible" r:id="rId509"/>
+    <sheet name="NetworkSecurityProtocols" sheetId="510" state="visible" r:id="rId510"/>
+    <sheet name="NonPersonalData" sheetId="511" state="visible" r:id="rId511"/>
+    <sheet name="Notification" sheetId="512" state="visible" r:id="rId512"/>
+    <sheet name="ObservedData" sheetId="513" state="visible" r:id="rId513"/>
+    <sheet name="ObservedPersonalData" sheetId="514" state="visible" r:id="rId514"/>
+    <sheet name="OperatingSystemSecurity" sheetId="515" state="visible" r:id="rId515"/>
+    <sheet name="PasswordAuthentication" sheetId="516" state="visible" r:id="rId516"/>
+    <sheet name="PenetrationTestingMethods" sheetId="517" state="visible" r:id="rId517"/>
+    <sheet name="PermissionManagement" sheetId="518" state="visible" r:id="rId518"/>
+    <sheet name="PersonalData" sheetId="519" state="visible" r:id="rId519"/>
+    <sheet name="PersonalDataAudit" sheetId="520" state="visible" r:id="rId520"/>
+    <sheet name="PhysicalAccessControlMethod" sheetId="521" state="visible" r:id="rId521"/>
+    <sheet name="PhysicalAuthentication" sheetId="522" state="visible" r:id="rId522"/>
+    <sheet name="PhysicalAuthorisation" sheetId="523" state="visible" r:id="rId523"/>
+    <sheet name="PhysicalDeviceSecurity" sheetId="524" state="visible" r:id="rId524"/>
+    <sheet name="PhysicalInterceptionProtection" sheetId="525" state="visible" r:id="rId525"/>
+    <sheet name="PhysicalInterruptionProtection" sheetId="526" state="visible" r:id="rId526"/>
+    <sheet name="PhysicalNetworkSecurity" sheetId="527" state="visible" r:id="rId527"/>
+    <sheet name="PhysicalSecureStorage" sheetId="528" state="visible" r:id="rId528"/>
+    <sheet name="PhysicalSupplySecurity" sheetId="529" state="visible" r:id="rId529"/>
+    <sheet name="PhysicalSurveillance" sheetId="530" state="visible" r:id="rId530"/>
+    <sheet name="Policy" sheetId="531" state="visible" r:id="rId531"/>
+    <sheet name="PostQuantumCryptography" sheetId="532" state="visible" r:id="rId532"/>
+    <sheet name="Principle" sheetId="533" state="visible" r:id="rId533"/>
+    <sheet name="PrivacyByDefault" sheetId="534" state="visible" r:id="rId534"/>
+    <sheet name="PrivacyByDesign" sheetId="535" state="visible" r:id="rId535"/>
+    <sheet name="PrivacyPreservingProtocol" sheetId="536" state="visible" r:id="rId536"/>
+    <sheet name="PrivateInformationRetrieval" sheetId="537" state="visible" r:id="rId537"/>
+    <sheet name="ProfessionalConfidentialData" sheetId="538" state="visible" r:id="rId538"/>
+    <sheet name="ProfessionalTraining" sheetId="539" state="visible" r:id="rId539"/>
+    <sheet name="ProvidedData" sheetId="540" state="visible" r:id="rId540"/>
+    <sheet name="ProvidedPersonalData" sheetId="541" state="visible" r:id="rId541"/>
+    <sheet name="Pseudonymisation" sheetId="542" state="visible" r:id="rId542"/>
+    <sheet name="PseudonymisedData" sheetId="543" state="visible" r:id="rId543"/>
+    <sheet name="QuantumCryptography" sheetId="544" state="visible" r:id="rId544"/>
+    <sheet name="RNGPseudonymisation" sheetId="545" state="visible" r:id="rId545"/>
+    <sheet name="ROPA" sheetId="546" state="visible" r:id="rId546"/>
+    <sheet name="RecertificationPolicy" sheetId="547" state="visible" r:id="rId547"/>
+    <sheet name="RecordsOfActivities" sheetId="548" state="visible" r:id="rId548"/>
+    <sheet name="RegulatorySandbox" sheetId="549" state="visible" r:id="rId549"/>
+    <sheet name="ReviewImpactAssessment" sheetId="550" state="visible" r:id="rId550"/>
+    <sheet name="ReviewProcedure" sheetId="551" state="visible" r:id="rId551"/>
+    <sheet name="RightsManagement" sheetId="552" state="visible" r:id="rId552"/>
+    <sheet name="Safeguard" sheetId="553" state="visible" r:id="rId553"/>
+    <sheet name="SafeguardForDataTransfer" sheetId="554" state="visible" r:id="rId554"/>
+    <sheet name="Seal" sheetId="555" state="visible" r:id="rId555"/>
+    <sheet name="SecretSharingSchemes" sheetId="556" state="visible" r:id="rId556"/>
+    <sheet name="SecureMultiPartyComputation" sheetId="557" state="visible" r:id="rId557"/>
+    <sheet name="SecureProcessingEnvironment" sheetId="558" state="visible" r:id="rId558"/>
+    <sheet name="SecurityAudit" sheetId="559" state="visible" r:id="rId559"/>
+    <sheet name="SecurityIncidentNotification" sheetId="560" state="visible" r:id="rId560"/>
+    <sheet name="SecurityIncidentRecord" sheetId="561" state="visible" r:id="rId561"/>
+    <sheet name="SecurityKnowledgeTraining" sheetId="562" state="visible" r:id="rId562"/>
+    <sheet name="SecurityMethod" sheetId="563" state="visible" r:id="rId563"/>
+    <sheet name="SecurityProcedure" sheetId="564" state="visible" r:id="rId564"/>
+    <sheet name="SecurityRoleProcedures" sheetId="565" state="visible" r:id="rId565"/>
+    <sheet name="SensitiveData" sheetId="566" state="visible" r:id="rId566"/>
+    <sheet name="SensitiveNonPersonalData" sheetId="567" state="visible" r:id="rId567"/>
+    <sheet name="SensitivePersonalData" sheetId="568" state="visible" r:id="rId568"/>
+    <sheet name="SingleSignOn" sheetId="569" state="visible" r:id="rId569"/>
+    <sheet name="SpecialCategoryPersonalData" sheetId="570" state="visible" r:id="rId570"/>
+    <sheet name="StaffTraining" sheetId="571" state="visible" r:id="rId571"/>
+    <sheet name="Standard" sheetId="572" state="visible" r:id="rId572"/>
+    <sheet name="StandardsConformance" sheetId="573" state="visible" r:id="rId573"/>
+    <sheet name="StatisticallyConfidentialData" sheetId="574" state="visible" r:id="rId574"/>
+    <sheet name="SupportContractNegotiation" sheetId="575" state="visible" r:id="rId575"/>
+    <sheet name="SupportEntityDecisionMaking" sheetId="576" state="visible" r:id="rId576"/>
+    <sheet name="SupportExchangeOfViews" sheetId="577" state="visible" r:id="rId577"/>
+    <sheet name="SupportInformedConsentDecision" sheetId="578" state="visible" r:id="rId578"/>
+    <sheet name="SymmetricCryptography" sheetId="579" state="visible" r:id="rId579"/>
+    <sheet name="SymmetricEncryption" sheetId="580" state="visible" r:id="rId580"/>
+    <sheet name="SyntheticData" sheetId="581" state="visible" r:id="rId581"/>
+    <sheet name="TechnicalStandard" sheetId="582" state="visible" r:id="rId582"/>
+    <sheet name="ThirdPartySecurityProcedures" sheetId="583" state="visible" r:id="rId583"/>
+    <sheet name="TrustedComputing" sheetId="584" state="visible" r:id="rId584"/>
+    <sheet name="TrustedExecutionEnvironment" sheetId="585" state="visible" r:id="rId585"/>
+    <sheet name="UncategorisedData" sheetId="586" state="visible" r:id="rId586"/>
+    <sheet name="UnstructuredData" sheetId="587" state="visible" r:id="rId587"/>
+    <sheet name="UnverifiedData" sheetId="588" state="visible" r:id="rId588"/>
+    <sheet name="UsageControl" sheetId="589" state="visible" r:id="rId589"/>
+    <sheet name="UseSyntheticData" sheetId="590" state="visible" r:id="rId590"/>
+    <sheet name="VerifiedData" sheetId="591" state="visible" r:id="rId591"/>
+    <sheet name="VirtualisationSecurity" sheetId="592" state="visible" r:id="rId592"/>
+    <sheet name="VulnerabilityTestingMethods" sheetId="593" state="visible" r:id="rId593"/>
+    <sheet name="WebBrowserSecurity" sheetId="594" state="visible" r:id="rId594"/>
+    <sheet name="WebSecurityProtocols" sheetId="595" state="visible" r:id="rId595"/>
+    <sheet name="WirelessSecurityProtocols" sheetId="596" state="visible" r:id="rId596"/>
+    <sheet name="ZeroKnowledgeAuthentication" sheetId="597" state="visible" r:id="rId597"/>
+    <sheet name="AcademicResearch" sheetId="598" state="visible" r:id="rId598"/>
+    <sheet name="Access" sheetId="599" state="visible" r:id="rId599"/>
+    <sheet name="AccountManagement" sheetId="600" state="visible" r:id="rId600"/>
+    <sheet name="Acquire" sheetId="601" state="visible" r:id="rId601"/>
+    <sheet name="Adapt" sheetId="602" state="visible" r:id="rId602"/>
+    <sheet name="Advertising" sheetId="603" state="visible" r:id="rId603"/>
+    <sheet name="AgeVerification" sheetId="604" state="visible" r:id="rId604"/>
+    <sheet name="Aggregate" sheetId="605" state="visible" r:id="rId605"/>
+    <sheet name="AlgorithmicLogic" sheetId="606" state="visible" r:id="rId606"/>
+    <sheet name="Align" sheetId="607" state="visible" r:id="rId607"/>
+    <sheet name="Alter" sheetId="608" state="visible" r:id="rId608"/>
+    <sheet name="Analyse" sheetId="609" state="visible" r:id="rId609"/>
+    <sheet name="Anonymise" sheetId="610" state="visible" r:id="rId610"/>
+    <sheet name="Assess" sheetId="611" state="visible" r:id="rId611"/>
+    <sheet name="AssistiveAutomation" sheetId="612" state="visible" r:id="rId612"/>
+    <sheet name="AutomatedDecisionMaking" sheetId="613" state="visible" r:id="rId613"/>
+    <sheet name="AutomatedScoringOfIndividuals" sheetId="614" state="visible" r:id="rId614"/>
+    <sheet name="AutomationLevel" sheetId="615" state="visible" r:id="rId615"/>
+    <sheet name="Autonomous" sheetId="616" state="visible" r:id="rId616"/>
+    <sheet name="CannotChallengeProcess" sheetId="617" state="visible" r:id="rId617"/>
+    <sheet name="CannotChallengeProcessInput" sheetId="618" state="visible" r:id="rId618"/>
+    <sheet name="CannotChallengeProcessOutput" sheetId="619" state="visible" r:id="rId619"/>
+    <sheet name="CannotCorrectProcess" sheetId="620" state="visible" r:id="rId620"/>
+    <sheet name="CannotCorrectProcessInput" sheetId="621" state="visible" r:id="rId621"/>
+    <sheet name="CannotCorrectProcessOutput" sheetId="622" state="visible" r:id="rId622"/>
+    <sheet name="CannotObjectToProcess" sheetId="623" state="visible" r:id="rId623"/>
+    <sheet name="CannotOptInToProcess" sheetId="624" state="visible" r:id="rId624"/>
+    <sheet name="CannotOptOutFromProcess" sheetId="625" state="visible" r:id="rId625"/>
+    <sheet name="CannotReverseProcessEffects" sheetId="626" state="visible" r:id="rId626"/>
+    <sheet name="CannotReverseProcessInput" sheetId="627" state="visible" r:id="rId627"/>
+    <sheet name="CannotReverseProcessOutput" sheetId="628" state="visible" r:id="rId628"/>
+    <sheet name="CannotWithdrawFromProcess" sheetId="629" state="visible" r:id="rId629"/>
+    <sheet name="ChallengingProcess" sheetId="630" state="visible" r:id="rId630"/>
+    <sheet name="ChallengingProcessInput" sheetId="631" state="visible" r:id="rId631"/>
+    <sheet name="ChallengingProcessOutput" sheetId="632" state="visible" r:id="rId632"/>
+    <sheet name="Collect" sheetId="633" state="visible" r:id="rId633"/>
+    <sheet name="CombatClimateChange" sheetId="634" state="visible" r:id="rId634"/>
+    <sheet name="Combine" sheetId="635" state="visible" r:id="rId635"/>
+    <sheet name="CommercialPurpose" sheetId="636" state="visible" r:id="rId636"/>
+    <sheet name="CommercialResearch" sheetId="637" state="visible" r:id="rId637"/>
+    <sheet name="CommunicationForCustomerCare" sheetId="638" state="visible" r:id="rId638"/>
+    <sheet name="CommunicationManagement" sheetId="639" state="visible" r:id="rId639"/>
+    <sheet name="ConditionalAutomation" sheetId="640" state="visible" r:id="rId640"/>
+    <sheet name="Consult" sheetId="641" state="visible" r:id="rId641"/>
+    <sheet name="Copy" sheetId="642" state="visible" r:id="rId642"/>
+    <sheet name="CorrectingProcess" sheetId="643" state="visible" r:id="rId643"/>
+    <sheet name="CorrectingProcessInput" sheetId="644" state="visible" r:id="rId644"/>
+    <sheet name="CorrectingProcessOutput" sheetId="645" state="visible" r:id="rId645"/>
+    <sheet name="CounterMoneyLaundering" sheetId="646" state="visible" r:id="rId646"/>
+    <sheet name="Counterterrorism" sheetId="647" state="visible" r:id="rId647"/>
+    <sheet name="CrossBorderTransfer" sheetId="648" state="visible" r:id="rId648"/>
+    <sheet name="CustomerCare" sheetId="649" state="visible" r:id="rId649"/>
+    <sheet name="CustomerClaimsManagement" sheetId="650" state="visible" r:id="rId650"/>
+    <sheet name="CustomerManagement" sheetId="651" state="visible" r:id="rId651"/>
+    <sheet name="CustomerOrderManagement" sheetId="652" state="visible" r:id="rId652"/>
+    <sheet name="CustomerRelationshipManagement" sheetId="653" state="visible" r:id="rId653"/>
+    <sheet name="CustomerSolvencyMonitoring" sheetId="654" state="visible" r:id="rId654"/>
+    <sheet name="DataAltruism" sheetId="655" state="visible" r:id="rId655"/>
+    <sheet name="DataControllerDataSource" sheetId="656" state="visible" r:id="rId656"/>
+    <sheet name="DataPublishedByDataSubject" sheetId="657" state="visible" r:id="rId657"/>
+    <sheet name="DataSource" sheetId="658" state="visible" r:id="rId658"/>
+    <sheet name="DataSubjectDataSource" sheetId="659" state="visible" r:id="rId659"/>
+    <sheet name="DataSubjectScale" sheetId="660" state="visible" r:id="rId660"/>
+    <sheet name="DataVolume" sheetId="661" state="visible" r:id="rId661"/>
+    <sheet name="DecisionMaking" sheetId="662" state="visible" r:id="rId662"/>
+    <sheet name="Delete" sheetId="663" state="visible" r:id="rId663"/>
+    <sheet name="DeliveryOfGoods" sheetId="664" state="visible" r:id="rId664"/>
+    <sheet name="Derive" sheetId="665" state="visible" r:id="rId665"/>
+    <sheet name="Destruct" sheetId="666" state="visible" r:id="rId666"/>
+    <sheet name="DirectMarketing" sheetId="667" state="visible" r:id="rId667"/>
+    <sheet name="Disclose" sheetId="668" state="visible" r:id="rId668"/>
+    <sheet name="DiscloseByTransmission" sheetId="669" state="visible" r:id="rId669"/>
+    <sheet name="Display" sheetId="670" state="visible" r:id="rId670"/>
+    <sheet name="DisputeManagement" sheetId="671" state="visible" r:id="rId671"/>
+    <sheet name="Disseminate" sheetId="672" state="visible" r:id="rId672"/>
+    <sheet name="Download" sheetId="673" state="visible" r:id="rId673"/>
+    <sheet name="DpvProcess" sheetId="674" state="visible" r:id="rId674"/>
+    <sheet name="DpvRecord" sheetId="675" state="visible" r:id="rId675"/>
+    <sheet name="DpvService" sheetId="676" state="visible" r:id="rId676"/>
+    <sheet name="EnforceAccessControl" sheetId="677" state="visible" r:id="rId677"/>
+    <sheet name="EnforceSecurity" sheetId="678" state="visible" r:id="rId678"/>
+    <sheet name="EntityActiveInvolvement" sheetId="679" state="visible" r:id="rId679"/>
+    <sheet name="EntityIntendedInvolvement" sheetId="680" state="visible" r:id="rId680"/>
+    <sheet name="EntityInvolved" sheetId="681" state="visible" r:id="rId681"/>
+    <sheet name="EntityInvolvement" sheetId="682" state="visible" r:id="rId682"/>
+    <sheet name="EntityInvolvementStatus" sheetId="683" state="visible" r:id="rId683"/>
+    <sheet name="EntityNonInvolvement" sheetId="684" state="visible" r:id="rId684"/>
+    <sheet name="EntityNonPermissiveInvolvement" sheetId="685" state="visible" r:id="rId685"/>
+    <sheet name="EntityNotInvolved" sheetId="686" state="visible" r:id="rId686"/>
+    <sheet name="EntityPassiveInvolvement" sheetId="687" state="visible" r:id="rId687"/>
+    <sheet name="EntityPermissiveInvolvement" sheetId="688" state="visible" r:id="rId688"/>
+    <sheet name="EntityUnintendedInvolvement" sheetId="689" state="visible" r:id="rId689"/>
+    <sheet name="Erase" sheetId="690" state="visible" r:id="rId690"/>
+    <sheet name="EstablishContractualAgreement" sheetId="691" state="visible" r:id="rId691"/>
+    <sheet name="EvaluationOfIndividuals" sheetId="692" state="visible" r:id="rId692"/>
+    <sheet name="EvaluationScoring" sheetId="693" state="visible" r:id="rId693"/>
+    <sheet name="Export" sheetId="694" state="visible" r:id="rId694"/>
+    <sheet name="Filter" sheetId="695" state="visible" r:id="rId695"/>
+    <sheet name="Format" sheetId="696" state="visible" r:id="rId696"/>
+    <sheet name="FraudPreventionAndDetection" sheetId="697" state="visible" r:id="rId697"/>
+    <sheet name="FulfilmentOfContractualObligation" sheetId="698" state="visible" r:id="rId698"/>
+    <sheet name="FulfilmentOfObligation" sheetId="699" state="visible" r:id="rId699"/>
+    <sheet name="FullAutomation" sheetId="700" state="visible" r:id="rId700"/>
+    <sheet name="Generate" sheetId="701" state="visible" r:id="rId701"/>
+    <sheet name="GeographicCoverage" sheetId="702" state="visible" r:id="rId702"/>
+    <sheet name="GlobalScale" sheetId="703" state="visible" r:id="rId703"/>
+    <sheet name="HighAutomation" sheetId="704" state="visible" r:id="rId704"/>
+    <sheet name="HugeDataVolume" sheetId="705" state="visible" r:id="rId705"/>
+    <sheet name="HugeScaleOfDataSubjects" sheetId="706" state="visible" r:id="rId706"/>
+    <sheet name="HumanInvolved" sheetId="707" state="visible" r:id="rId707"/>
+    <sheet name="HumanInvolvement" sheetId="708" state="visible" r:id="rId708"/>
+    <sheet name="HumanInvolvementForControl" sheetId="709" state="visible" r:id="rId709"/>
+    <sheet name="HumanInvolvementForDecision" sheetId="710" state="visible" r:id="rId710"/>
+    <sheet name="HumanInvolvementForInput" sheetId="711" state="visible" r:id="rId711"/>
+    <sheet name="HumanInvolvementForIntervention" sheetId="712" state="visible" r:id="rId712"/>
+    <sheet name="HumanInvolvementForOversight" sheetId="713" state="visible" r:id="rId713"/>
+    <sheet name="HumanInvolvementForVerification" sheetId="714" state="visible" r:id="rId714"/>
+    <sheet name="HumanNotInvolved" sheetId="715" state="visible" r:id="rId715"/>
+    <sheet name="HumanResourceManagement" sheetId="716" state="visible" r:id="rId716"/>
+    <sheet name="IdentityAuthentication" sheetId="717" state="visible" r:id="rId717"/>
+    <sheet name="IdentityVerification" sheetId="718" state="visible" r:id="rId718"/>
+    <sheet name="ImproveExistingProductsAndServices" sheetId="719" state="visible" r:id="rId719"/>
+    <sheet name="ImproveHealthcare" sheetId="720" state="visible" r:id="rId720"/>
+    <sheet name="ImproveInternalCRMProcesses" sheetId="721" state="visible" r:id="rId721"/>
+    <sheet name="ImprovePublicServices" sheetId="722" state="visible" r:id="rId722"/>
+    <sheet name="ImproveTransportMobility" sheetId="723" state="visible" r:id="rId723"/>
+    <sheet name="IncreaseServiceRobustness" sheetId="724" state="visible" r:id="rId724"/>
+    <sheet name="Infer" sheetId="725" state="visible" r:id="rId725"/>
+    <sheet name="InnovativeUseOfExistingTechnology" sheetId="726" state="visible" r:id="rId726"/>
+    <sheet name="InnovativeUseOfNewTechnologies" sheetId="727" state="visible" r:id="rId727"/>
+    <sheet name="InnovativeUseOfTechnology" sheetId="728" state="visible" r:id="rId728"/>
+    <sheet name="InternalResourceOptimisation" sheetId="729" state="visible" r:id="rId729"/>
+    <sheet name="LargeDataVolume" sheetId="730" state="visible" r:id="rId730"/>
+    <sheet name="LargeScaleOfDataSubjects" sheetId="731" state="visible" r:id="rId731"/>
+    <sheet name="LargeScaleProcessing" sheetId="732" state="visible" r:id="rId732"/>
+    <sheet name="LegalCompliance" sheetId="733" state="visible" r:id="rId733"/>
+    <sheet name="LocalEnvironmentScale" sheetId="734" state="visible" r:id="rId734"/>
+    <sheet name="LocalityScale" sheetId="735" state="visible" r:id="rId735"/>
+    <sheet name="MaintainFraudDatabase" sheetId="736" state="visible" r:id="rId736"/>
+    <sheet name="MakeAvailable" sheetId="737" state="visible" r:id="rId737"/>
+    <sheet name="Marketing" sheetId="738" state="visible" r:id="rId738"/>
+    <sheet name="Match" sheetId="739" state="visible" r:id="rId739"/>
+    <sheet name="MediumDataVolume" sheetId="740" state="visible" r:id="rId740"/>
+    <sheet name="MediumScaleOfDataSubjects" sheetId="741" state="visible" r:id="rId741"/>
+    <sheet name="MediumScaleProcessing" sheetId="742" state="visible" r:id="rId742"/>
+    <sheet name="MemberPartnerManagement" sheetId="743" state="visible" r:id="rId743"/>
+    <sheet name="MisusePreventionAndDetection" sheetId="744" state="visible" r:id="rId744"/>
+    <sheet name="Modify" sheetId="745" state="visible" r:id="rId745"/>
+    <sheet name="Monitor" sheetId="746" state="visible" r:id="rId746"/>
+    <sheet name="Move" sheetId="747" state="visible" r:id="rId747"/>
+    <sheet name="MultiNationalScale" sheetId="748" state="visible" r:id="rId748"/>
+    <sheet name="NationalScale" sheetId="749" state="visible" r:id="rId749"/>
+    <sheet name="NearlyGlobalScale" sheetId="750" state="visible" r:id="rId750"/>
+    <sheet name="NonCommercialPurpose" sheetId="751" state="visible" r:id="rId751"/>
+    <sheet name="NonCommercialResearch" sheetId="752" state="visible" r:id="rId752"/>
+    <sheet name="NonPersonalDataProcess" sheetId="753" state="visible" r:id="rId753"/>
+    <sheet name="NonPublicDataSource" sheetId="754" state="visible" r:id="rId754"/>
+    <sheet name="NotAutomated" sheetId="755" state="visible" r:id="rId755"/>
+    <sheet name="ObjectingToProcess" sheetId="756" state="visible" r:id="rId756"/>
+    <sheet name="Observe" sheetId="757" state="visible" r:id="rId757"/>
+    <sheet name="Obtain" sheetId="758" state="visible" r:id="rId758"/>
+    <sheet name="OptimisationForConsumer" sheetId="759" state="visible" r:id="rId759"/>
+    <sheet name="OptimisationForController" sheetId="760" state="visible" r:id="rId760"/>
+    <sheet name="OptimiseUserInterface" sheetId="761" state="visible" r:id="rId761"/>
+    <sheet name="OptingInToProcess" sheetId="762" state="visible" r:id="rId762"/>
+    <sheet name="OptingOutFromProcess" sheetId="763" state="visible" r:id="rId763"/>
+    <sheet name="OrganisationComplianceManagement" sheetId="764" state="visible" r:id="rId764"/>
+    <sheet name="OrganisationGovernance" sheetId="765" state="visible" r:id="rId765"/>
+    <sheet name="OrganisationRiskManagement" sheetId="766" state="visible" r:id="rId766"/>
+    <sheet name="Organise" sheetId="767" state="visible" r:id="rId767"/>
+    <sheet name="PartialAutomation" sheetId="768" state="visible" r:id="rId768"/>
+    <sheet name="PaymentManagement" sheetId="769" state="visible" r:id="rId769"/>
+    <sheet name="PersonalDataHandling" sheetId="770" state="visible" r:id="rId770"/>
+    <sheet name="PersonalDataProcess" sheetId="771" state="visible" r:id="rId771"/>
+    <sheet name="Personalisation" sheetId="772" state="visible" r:id="rId772"/>
+    <sheet name="PersonalisedAdvertising" sheetId="773" state="visible" r:id="rId773"/>
+    <sheet name="PersonalisedBenefits" sheetId="774" state="visible" r:id="rId774"/>
+    <sheet name="PersonnelBehaviourMonitoring" sheetId="775" state="visible" r:id="rId775"/>
+    <sheet name="PersonnelHiring" sheetId="776" state="visible" r:id="rId776"/>
+    <sheet name="PersonnelManagement" sheetId="777" state="visible" r:id="rId777"/>
+    <sheet name="PersonnelMonitoring" sheetId="778" state="visible" r:id="rId778"/>
+    <sheet name="PersonnelOffboarding" sheetId="779" state="visible" r:id="rId779"/>
+    <sheet name="PersonnelOnboarding" sheetId="780" state="visible" r:id="rId780"/>
+    <sheet name="PersonnelPayment" sheetId="781" state="visible" r:id="rId781"/>
+    <sheet name="PersonnelPerformanceEvaluation" sheetId="782" state="visible" r:id="rId782"/>
+    <sheet name="PersonnelPerformanceManagement" sheetId="783" state="visible" r:id="rId783"/>
+    <sheet name="PersonnelPerformanceMonitoring" sheetId="784" state="visible" r:id="rId784"/>
+    <sheet name="PersonnelPerformancePrediction" sheetId="785" state="visible" r:id="rId785"/>
+    <sheet name="PersonnelPromotionManagement" sheetId="786" state="visible" r:id="rId786"/>
+    <sheet name="PersonnelTerminationManagement" sheetId="787" state="visible" r:id="rId787"/>
+    <sheet name="PersonnelWorkloadManagement" sheetId="788" state="visible" r:id="rId788"/>
+    <sheet name="PoliticalCampaign" sheetId="789" state="visible" r:id="rId789"/>
+    <sheet name="Processing" sheetId="790" state="visible" r:id="rId790"/>
+    <sheet name="ProcessingCondition" sheetId="791" state="visible" r:id="rId791"/>
+    <sheet name="ProcessingContext" sheetId="792" state="visible" r:id="rId792"/>
+    <sheet name="ProcessingDuration" sheetId="793" state="visible" r:id="rId793"/>
+    <sheet name="ProcessingLocation" sheetId="794" state="visible" r:id="rId794"/>
+    <sheet name="ProcessingScale" sheetId="795" state="visible" r:id="rId795"/>
+    <sheet name="Profiling" sheetId="796" state="visible" r:id="rId796"/>
+    <sheet name="ProtectionOfIPR" sheetId="797" state="visible" r:id="rId797"/>
+    <sheet name="ProtectionOfNationalSecurity" sheetId="798" state="visible" r:id="rId798"/>
+    <sheet name="ProtectionOfPublicSecurity" sheetId="799" state="visible" r:id="rId799"/>
+    <sheet name="ProvideEventRecommendations" sheetId="800" state="visible" r:id="rId800"/>
+    <sheet name="ProvideOfficialStatistics" sheetId="801" state="visible" r:id="rId801"/>
+    <sheet name="ProvidePersonalisedRecommendations" sheetId="802" state="visible" r:id="rId802"/>
+    <sheet name="ProvideProductRecommendations" sheetId="803" state="visible" r:id="rId803"/>
+    <sheet name="Pseudonymise" sheetId="804" state="visible" r:id="rId804"/>
+    <sheet name="PublicBenefit" sheetId="805" state="visible" r:id="rId805"/>
+    <sheet name="PublicDataSource" sheetId="806" state="visible" r:id="rId806"/>
+    <sheet name="PublicPolicyMaking" sheetId="807" state="visible" r:id="rId807"/>
+    <sheet name="PublicRelations" sheetId="808" state="visible" r:id="rId808"/>
+    <sheet name="Purpose" sheetId="809" state="visible" r:id="rId809"/>
+    <sheet name="Query" sheetId="810" state="visible" r:id="rId810"/>
+    <sheet name="RecordManagement" sheetId="811" state="visible" r:id="rId811"/>
+    <sheet name="RecruitmentAdvertising" sheetId="812" state="visible" r:id="rId812"/>
+    <sheet name="RecruitmentApplicantBackgroundCheck" sheetId="813" state="visible" r:id="rId813"/>
+    <sheet name="RecruitmentApplicantCriminalBackgroundCheck" sheetId="814" state="visible" r:id="rId814"/>
+    <sheet name="RecruitmentApplicantInformationAuthentication" sheetId="815" state="visible" r:id="rId815"/>
+    <sheet name="RecruitmentApplicantSelection" sheetId="816" state="visible" r:id="rId816"/>
+    <sheet name="RecruitmentApplicationAnalysis" sheetId="817" state="visible" r:id="rId817"/>
+    <sheet name="RecruitmentApplicationManagement" sheetId="818" state="visible" r:id="rId818"/>
+    <sheet name="RecruitmentApplicationScreening" sheetId="819" state="visible" r:id="rId819"/>
+    <sheet name="RecruitmentInterviewAnalysis" sheetId="820" state="visible" r:id="rId820"/>
+    <sheet name="RecruitmentInterviewAssessment" sheetId="821" state="visible" r:id="rId821"/>
+    <sheet name="RecruitmentInterviewManagement" sheetId="822" state="visible" r:id="rId822"/>
+    <sheet name="RecruitmentInterviewScheduling" sheetId="823" state="visible" r:id="rId823"/>
+    <sheet name="RecruitmentManagement" sheetId="824" state="visible" r:id="rId824"/>
+    <sheet name="RecruitmentTargetedAdvertising" sheetId="825" state="visible" r:id="rId825"/>
+    <sheet name="Reformat" sheetId="826" state="visible" r:id="rId826"/>
+    <sheet name="RegionalScale" sheetId="827" state="visible" r:id="rId827"/>
+    <sheet name="Remove" sheetId="828" state="visible" r:id="rId828"/>
+    <sheet name="RepairImpairments" sheetId="829" state="visible" r:id="rId829"/>
+    <sheet name="RequestedServiceProvision" sheetId="830" state="visible" r:id="rId830"/>
+    <sheet name="ResearchAndDevelopment" sheetId="831" state="visible" r:id="rId831"/>
+    <sheet name="Restrict" sheetId="832" state="visible" r:id="rId832"/>
+    <sheet name="Retrieve" sheetId="833" state="visible" r:id="rId833"/>
+    <sheet name="ReversingProcessEffects" sheetId="834" state="visible" r:id="rId834"/>
+    <sheet name="ReversingProcessInput" sheetId="835" state="visible" r:id="rId835"/>
+    <sheet name="ReversingProcessOutput" sheetId="836" state="visible" r:id="rId836"/>
+    <sheet name="RightsFulfilment" sheetId="837" state="visible" r:id="rId837"/>
+    <sheet name="Scale" sheetId="838" state="visible" r:id="rId838"/>
+    <sheet name="ScientificResearch" sheetId="839" state="visible" r:id="rId839"/>
+    <sheet name="ScoringOfIndividuals" sheetId="840" state="visible" r:id="rId840"/>
+    <sheet name="Screen" sheetId="841" state="visible" r:id="rId841"/>
+    <sheet name="SearchFunctionalities" sheetId="842" state="visible" r:id="rId842"/>
+    <sheet name="Sector" sheetId="843" state="visible" r:id="rId843"/>
+    <sheet name="SellDataToThirdParties" sheetId="844" state="visible" r:id="rId844"/>
+    <sheet name="SellInsightsFromData" sheetId="845" state="visible" r:id="rId845"/>
+    <sheet name="SellProducts" sheetId="846" state="visible" r:id="rId846"/>
+    <sheet name="SellProductsToDataSubject" sheetId="847" state="visible" r:id="rId847"/>
+    <sheet name="ServiceAccessDetermination" sheetId="848" state="visible" r:id="rId848"/>
+    <sheet name="ServiceManagement" sheetId="849" state="visible" r:id="rId849"/>
+    <sheet name="ServiceMonitoring" sheetId="850" state="visible" r:id="rId850"/>
+    <sheet name="ServiceOptimisation" sheetId="851" state="visible" r:id="rId851"/>
+    <sheet name="ServicePersonalisation" sheetId="852" state="visible" r:id="rId852"/>
+    <sheet name="ServiceProvision" sheetId="853" state="visible" r:id="rId853"/>
+    <sheet name="ServiceRegistration" sheetId="854" state="visible" r:id="rId854"/>
+    <sheet name="ServiceUsageAnalytics" sheetId="855" state="visible" r:id="rId855"/>
+    <sheet name="Share" sheetId="856" state="visible" r:id="rId856"/>
+    <sheet name="SingularDataVolume" sheetId="857" state="visible" r:id="rId857"/>
+    <sheet name="SingularScaleOfDataSubjects" sheetId="858" state="visible" r:id="rId858"/>
+    <sheet name="SmallDataVolume" sheetId="859" state="visible" r:id="rId859"/>
+    <sheet name="SmallScaleOfDataSubjects" sheetId="860" state="visible" r:id="rId860"/>
+    <sheet name="SmallScaleProcessing" sheetId="861" state="visible" r:id="rId861"/>
+    <sheet name="SocialMediaMarketing" sheetId="862" state="visible" r:id="rId862"/>
+    <sheet name="SporadicDataVolume" sheetId="863" state="visible" r:id="rId863"/>
+    <sheet name="SporadicScaleOfDataSubjects" sheetId="864" state="visible" r:id="rId864"/>
+    <sheet name="StorageCondition" sheetId="865" state="visible" r:id="rId865"/>
+    <sheet name="StorageDeletion" sheetId="866" state="visible" r:id="rId866"/>
+    <sheet name="StorageDuration" sheetId="867" state="visible" r:id="rId867"/>
+    <sheet name="StorageLocation" sheetId="868" state="visible" r:id="rId868"/>
+    <sheet name="StorageRestoration" sheetId="869" state="visible" r:id="rId869"/>
+    <sheet name="Store" sheetId="870" state="visible" r:id="rId870"/>
+    <sheet name="Structure" sheetId="871" state="visible" r:id="rId871"/>
+    <sheet name="SystematicMonitoring" sheetId="872" state="visible" r:id="rId872"/>
+    <sheet name="TargetedAdvertising" sheetId="873" state="visible" r:id="rId873"/>
+    <sheet name="TechnicalServiceProvision" sheetId="874" state="visible" r:id="rId874"/>
+    <sheet name="Technology" sheetId="875" state="visible" r:id="rId875"/>
+    <sheet name="ThirdPartyDataSource" sheetId="876" state="visible" r:id="rId876"/>
+    <sheet name="Tracking" sheetId="877" state="visible" r:id="rId877"/>
+    <sheet name="TrackingByFirstParty" sheetId="878" state="visible" r:id="rId878"/>
+    <sheet name="TrackingByThirdParty" sheetId="879" state="visible" r:id="rId879"/>
+    <sheet name="Transfer" sheetId="880" state="visible" r:id="rId880"/>
+    <sheet name="Transform" sheetId="881" state="visible" r:id="rId881"/>
+    <sheet name="Transmit" sheetId="882" state="visible" r:id="rId882"/>
+    <sheet name="Use" sheetId="883" state="visible" r:id="rId883"/>
+    <sheet name="UserInterfacePersonalisation" sheetId="884" state="visible" r:id="rId884"/>
+    <sheet name="VendorManagement" sheetId="885" state="visible" r:id="rId885"/>
+    <sheet name="VendorPayment" sheetId="886" state="visible" r:id="rId886"/>
+    <sheet name="VendorRecordsManagement" sheetId="887" state="visible" r:id="rId887"/>
+    <sheet name="VendorSelectionAssessment" sheetId="888" state="visible" r:id="rId888"/>
+    <sheet name="Verification" sheetId="889" state="visible" r:id="rId889"/>
+    <sheet name="WithdrawingFromProcess" sheetId="890" state="visible" r:id="rId890"/>
+    <sheet name="ConsentNotice" sheetId="891" state="visible" r:id="rId891"/>
+    <sheet name="Consequence" sheetId="892" state="visible" r:id="rId892"/>
+    <sheet name="ConsequenceAsSideEffect" sheetId="893" state="visible" r:id="rId893"/>
+    <sheet name="ConsequenceOfFailure" sheetId="894" state="visible" r:id="rId894"/>
+    <sheet name="ConsequenceOfSuccess" sheetId="895" state="visible" r:id="rId895"/>
+    <sheet name="CybersecurityAssessment" sheetId="896" state="visible" r:id="rId896"/>
+    <sheet name="DPIA" sheetId="897" state="visible" r:id="rId897"/>
+    <sheet name="DashboardNotice" sheetId="898" state="visible" r:id="rId898"/>
+    <sheet name="DataBreachImpactAssessment" sheetId="899" state="visible" r:id="rId899"/>
+    <sheet name="DataBreachNotice" sheetId="900" state="visible" r:id="rId900"/>
+    <sheet name="DataTransferImpactAssessment" sheetId="901" state="visible" r:id="rId901"/>
+    <sheet name="DataTransferNotice" sheetId="902" state="visible" r:id="rId902"/>
+    <sheet name="DeviceNotice" sheetId="903" state="visible" r:id="rId903"/>
+    <sheet name="FRIA" sheetId="904" state="visible" r:id="rId904"/>
+    <sheet name="GraphicalNotice" sheetId="905" state="visible" r:id="rId905"/>
+    <sheet name="Impact" sheetId="906" state="visible" r:id="rId906"/>
+    <sheet name="ImpactAssessment" sheetId="907" state="visible" r:id="rId907"/>
+    <sheet name="JITNotice" sheetId="908" state="visible" r:id="rId908"/>
+    <sheet name="LayeredNotice" sheetId="909" state="visible" r:id="rId909"/>
+    <sheet name="Likelihood" sheetId="910" state="visible" r:id="rId910"/>
+    <sheet name="Notice" sheetId="911" state="visible" r:id="rId911"/>
+    <sheet name="NoticeCommunicated" sheetId="912" state="visible" r:id="rId912"/>
+    <sheet name="NoticeGenerated" sheetId="913" state="visible" r:id="rId913"/>
+    <sheet name="NoticeIcon" sheetId="914" state="visible" r:id="rId914"/>
+    <sheet name="NoticeLatest" sheetId="915" state="visible" r:id="rId915"/>
+    <sheet name="NoticeLayer" sheetId="916" state="visible" r:id="rId916"/>
+    <sheet name="NoticeStale" sheetId="917" state="visible" r:id="rId917"/>
+    <sheet name="NoticeStatus" sheetId="918" state="visible" r:id="rId918"/>
+    <sheet name="NoticeUnused" sheetId="919" state="visible" r:id="rId919"/>
+    <sheet name="NoticeUpdated" sheetId="920" state="visible" r:id="rId920"/>
+    <sheet name="NoticeUsed" sheetId="921" state="visible" r:id="rId921"/>
+    <sheet name="OralNotice" sheetId="922" state="visible" r:id="rId922"/>
+    <sheet name="PIA" sheetId="923" state="visible" r:id="rId923"/>
+    <sheet name="PostedNotice" sheetId="924" state="visible" r:id="rId924"/>
+    <sheet name="PrintedNotice" sheetId="925" state="visible" r:id="rId925"/>
+    <sheet name="PrivacyNotice" sheetId="926" state="visible" r:id="rId926"/>
+    <sheet name="ResidualRisk" sheetId="927" state="visible" r:id="rId927"/>
+    <sheet name="RightsImpactAssessment" sheetId="928" state="visible" r:id="rId928"/>
+    <sheet name="Risk" sheetId="929" state="visible" r:id="rId929"/>
+    <sheet name="RiskAssessment" sheetId="930" state="visible" r:id="rId930"/>
+    <sheet name="RiskConcept" sheetId="931" state="visible" r:id="rId931"/>
+    <sheet name="RiskLevel" sheetId="932" state="visible" r:id="rId932"/>
+    <sheet name="RiskMitigationMeasure" sheetId="933" state="visible" r:id="rId933"/>
+    <sheet name="SecurityAssessment" sheetId="934" state="visible" r:id="rId934"/>
+    <sheet name="SecurityIncidentNotice" sheetId="935" state="visible" r:id="rId935"/>
+    <sheet name="SensitivityLevel" sheetId="936" state="visible" r:id="rId936"/>
+    <sheet name="Severity" sheetId="937" state="visible" r:id="rId937"/>
+    <sheet name="ActiveRight" sheetId="938" state="visible" r:id="rId938"/>
+    <sheet name="DataSubjectRight" sheetId="939" state="visible" r:id="rId939"/>
+    <sheet name="PassiveRight" sheetId="940" state="visible" r:id="rId940"/>
+    <sheet name="Right" sheetId="941" state="visible" r:id="rId941"/>
+    <sheet name="RightExerciseActivity" sheetId="942" state="visible" r:id="rId942"/>
+    <sheet name="RightExerciseNotice" sheetId="943" state="visible" r:id="rId943"/>
+    <sheet name="RightExerciseRecord" sheetId="944" state="visible" r:id="rId944"/>
+    <sheet name="RightFulfilmentNotice" sheetId="945" state="visible" r:id="rId945"/>
+    <sheet name="RightNonFulfilmentNotice" sheetId="946" state="visible" r:id="rId946"/>
+    <sheet name="RightNotice" sheetId="947" state="visible" r:id="rId947"/>
+    <sheet name="ConsentControl" sheetId="948" state="visible" r:id="rId948"/>
+    <sheet name="ConsentExpired" sheetId="949" state="visible" r:id="rId949"/>
+    <sheet name="ConsentGiven" sheetId="950" state="visible" r:id="rId950"/>
+    <sheet name="ConsentInvalidated" sheetId="951" state="visible" r:id="rId951"/>
+    <sheet name="ConsentRefused" sheetId="952" state="visible" r:id="rId952"/>
+    <sheet name="ConsentRequestDeferred" sheetId="953" state="visible" r:id="rId953"/>
+    <sheet name="ConsentRequested" sheetId="954" state="visible" r:id="rId954"/>
+    <sheet name="ConsentRevoked" sheetId="955" state="visible" r:id="rId955"/>
+    <sheet name="ConsentStatus" sheetId="956" state="visible" r:id="rId956"/>
+    <sheet name="ConsentStatusInvalidForProcessing" sheetId="957" state="visible" r:id="rId957"/>
+    <sheet name="ConsentStatusValidForProcessing" sheetId="958" state="visible" r:id="rId958"/>
+    <sheet name="ConsentUnknown" sheetId="959" state="visible" r:id="rId959"/>
+    <sheet name="ConsentWithdrawn" sheetId="960" state="visible" r:id="rId960"/>
+    <sheet name="ExplicitlyExpressedConsent" sheetId="961" state="visible" r:id="rId961"/>
+    <sheet name="ExpressedConsent" sheetId="962" state="visible" r:id="rId962"/>
+    <sheet name="ImpliedConsent" sheetId="963" state="visible" r:id="rId963"/>
+    <sheet name="InformedConsent" sheetId="964" state="visible" r:id="rId964"/>
+    <sheet name="ManageConsent" sheetId="965" state="visible" r:id="rId965"/>
+    <sheet name="ObtainConsent" sheetId="966" state="visible" r:id="rId966"/>
+    <sheet name="ProvideConsent" sheetId="967" state="visible" r:id="rId967"/>
+    <sheet name="ReaffirmConsent" sheetId="968" state="visible" r:id="rId968"/>
+    <sheet name="RefuseConsent" sheetId="969" state="visible" r:id="rId969"/>
+    <sheet name="RenewedConsentGiven" sheetId="970" state="visible" r:id="rId970"/>
+    <sheet name="UninformedConsent" sheetId="971" state="visible" r:id="rId971"/>
+    <sheet name="WithdrawConsent" sheetId="972" state="visible" r:id="rId972"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>